<commit_message>
changed stocks path extraction path
</commit_message>
<xml_diff>
--- a/data/ready_stocks/galtex-ozon-stocks-updated.xlsx
+++ b/data/ready_stocks/galtex-ozon-stocks-updated.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D186"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -418,13 +418,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B2" t="str">
-        <v>TMbeige140150</v>
+        <v>TG1VichyLightBlue220/33</v>
       </c>
       <c r="C2" t="str">
         <v/>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -432,7 +432,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B3" t="str">
-        <v>TMblue140150</v>
+        <v>TG1LabirintVasilek220/33</v>
       </c>
       <c r="C3" t="str">
         <v/>
@@ -446,7 +446,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B4" t="str">
-        <v>TMbordo140150</v>
+        <v>TG1TropicanaBeige220/33</v>
       </c>
       <c r="C4" t="str">
         <v/>
@@ -460,13 +460,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B5" t="str">
-        <v>TMbrown140150</v>
+        <v>TG1LondonTurquoise220/33</v>
       </c>
       <c r="C5" t="str">
         <v/>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
@@ -474,13 +474,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B6" t="str">
-        <v>TMgrey140150</v>
+        <v>TG1MramorTurquoise</v>
       </c>
       <c r="C6" t="str">
         <v/>
       </c>
       <c r="D6">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -488,7 +488,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B7" t="str">
-        <v>TMIzumrud140150</v>
+        <v>TG1MramorGrey</v>
       </c>
       <c r="C7" t="str">
         <v/>
@@ -502,7 +502,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B8" t="str">
-        <v>TMLightBlue140150</v>
+        <v>TG1ValenciaBlueLiliac</v>
       </c>
       <c r="C8" t="str">
         <v/>
@@ -516,13 +516,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B9" t="str">
-        <v>TMLightLilov140150</v>
+        <v>TG1MonblanColour</v>
       </c>
       <c r="C9" t="str">
         <v/>
       </c>
       <c r="D9">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
@@ -530,7 +530,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B10" t="str">
-        <v>TMLightViolet140150</v>
+        <v>TG1VoskhodOrange</v>
       </c>
       <c r="C10" t="str">
         <v/>
@@ -544,13 +544,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B11" t="str">
-        <v>TMOhra140150</v>
+        <v>TG1KaramelBZ</v>
       </c>
       <c r="C11" t="str">
         <v/>
       </c>
       <c r="D11">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12">
@@ -558,13 +558,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B12" t="str">
-        <v>TMPersik140150</v>
+        <v>TG1VichyBej</v>
       </c>
       <c r="C12" t="str">
         <v/>
       </c>
       <c r="D12">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13">
@@ -572,7 +572,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B13" t="str">
-        <v>TMpink140150</v>
+        <v>TG1RomanticBlue</v>
       </c>
       <c r="C13" t="str">
         <v/>
@@ -586,13 +586,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B14" t="str">
-        <v>TMred140150</v>
+        <v>TG1SymphonyGreyBej</v>
       </c>
       <c r="C14" t="str">
         <v/>
       </c>
       <c r="D14">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -600,7 +600,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B15" t="str">
-        <v>TMSalad140150</v>
+        <v>TG1ValenciaTurquoiseGreen</v>
       </c>
       <c r="C15" t="str">
         <v/>
@@ -614,7 +614,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B16" t="str">
-        <v>TMSeaWave140150</v>
+        <v>TG1TropicTurquoise</v>
       </c>
       <c r="C16" t="str">
         <v/>
@@ -628,13 +628,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B17" t="str">
-        <v>TMsilverGrey140150</v>
+        <v>TG1TropicanaBlack</v>
       </c>
       <c r="C17" t="str">
         <v/>
       </c>
       <c r="D17">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18">
@@ -642,7 +642,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B18" t="str">
-        <v>TMSvetloGoluboi140150</v>
+        <v>TG1TattersolGreyBej</v>
       </c>
       <c r="C18" t="str">
         <v/>
@@ -656,7 +656,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B19" t="str">
-        <v>TMViolet140150</v>
+        <v>TG1TreugLightBlue220/33</v>
       </c>
       <c r="C19" t="str">
         <v/>
@@ -670,7 +670,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B20" t="str">
-        <v>TMblack140150</v>
+        <v>TG1NiagaraTurquoise</v>
       </c>
       <c r="C20" t="str">
         <v/>
@@ -684,7 +684,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B21" t="str">
-        <v>TMcharcoal-grey140150</v>
+        <v>TG1NiagaraYellow</v>
       </c>
       <c r="C21" t="str">
         <v/>
@@ -698,7 +698,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B22" t="str">
-        <v>TMkakao140150</v>
+        <v>TG1Smiles</v>
       </c>
       <c r="C22" t="str">
         <v/>
@@ -712,18 +712,2300 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B23" t="str">
-        <v>TMoliva140150</v>
+        <v>TG1Aquarelle</v>
       </c>
       <c r="C23" t="str">
         <v/>
       </c>
       <c r="D23">
         <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B24" t="str">
+        <v>TG1BogemaTurquoise</v>
+      </c>
+      <c r="C24" t="str">
+        <v/>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B25" t="str">
+        <v>TG1MadlenGrey</v>
+      </c>
+      <c r="C25" t="str">
+        <v/>
+      </c>
+      <c r="D25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B26" t="str">
+        <v>TG1ZavitokChoco</v>
+      </c>
+      <c r="C26" t="str">
+        <v/>
+      </c>
+      <c r="D26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B27" t="str">
+        <v>TG1CubicBej</v>
+      </c>
+      <c r="C27" t="str">
+        <v/>
+      </c>
+      <c r="D27">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B28" t="str">
+        <v>TG1RomanticLightBlue</v>
+      </c>
+      <c r="C28" t="str">
+        <v/>
+      </c>
+      <c r="D28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B29" t="str">
+        <v>TG1ConfettiLime</v>
+      </c>
+      <c r="C29" t="str">
+        <v/>
+      </c>
+      <c r="D29">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B30" t="str">
+        <v>TG1Florans</v>
+      </c>
+      <c r="C30" t="str">
+        <v/>
+      </c>
+      <c r="D30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B31" t="str">
+        <v>TG1BeskonechnostBZ</v>
+      </c>
+      <c r="C31" t="str">
+        <v/>
+      </c>
+      <c r="D31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B32" t="str">
+        <v>TG1JungleGreyBej</v>
+      </c>
+      <c r="C32" t="str">
+        <v/>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B33" t="str">
+        <v>TG1BogemaGrey</v>
+      </c>
+      <c r="C33" t="str">
+        <v/>
+      </c>
+      <c r="D33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B34" t="str">
+        <v>TG1GraciaBZgrey</v>
+      </c>
+      <c r="C34" t="str">
+        <v/>
+      </c>
+      <c r="D34">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B35" t="str">
+        <v>TG2EucaliptusBlue220/33</v>
+      </c>
+      <c r="C35" t="str">
+        <v/>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B36" t="str">
+        <v>TG2WesternSeaWave220/33</v>
+      </c>
+      <c r="C36" t="str">
+        <v/>
+      </c>
+      <c r="D36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B37" t="str">
+        <v>TG2SonetBZ</v>
+      </c>
+      <c r="C37" t="str">
+        <v/>
+      </c>
+      <c r="D37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B38" t="str">
+        <v>TG2FlowersSakurPowder</v>
+      </c>
+      <c r="C38" t="str">
+        <v/>
+      </c>
+      <c r="D38">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B39" t="str">
+        <v>TG2DunovenieGreyBeige</v>
+      </c>
+      <c r="C39" t="str">
+        <v/>
+      </c>
+      <c r="D39">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B40" t="str">
+        <v>TG2ContourGreen</v>
+      </c>
+      <c r="C40" t="str">
+        <v/>
+      </c>
+      <c r="D40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B41" t="str">
+        <v>TG2LabirintBrown</v>
+      </c>
+      <c r="C41" t="str">
+        <v/>
+      </c>
+      <c r="D41">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B42" t="str">
+        <v>TG2WesternPowder</v>
+      </c>
+      <c r="C42" t="str">
+        <v/>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B43" t="str">
+        <v>TG2EverestDarkGrey</v>
+      </c>
+      <c r="C43" t="str">
+        <v/>
+      </c>
+      <c r="D43">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B44" t="str">
+        <v>TG2CreativeGreyBej</v>
+      </c>
+      <c r="C44" t="str">
+        <v/>
+      </c>
+      <c r="D44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B45" t="str">
+        <v>TG2ContourDarkGrey</v>
+      </c>
+      <c r="C45" t="str">
+        <v/>
+      </c>
+      <c r="D45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B46" t="str">
+        <v>TG2CollageBejBlue</v>
+      </c>
+      <c r="C46" t="str">
+        <v/>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B47" t="str">
+        <v>TG2SymphonyLightBlue</v>
+      </c>
+      <c r="C47" t="str">
+        <v/>
+      </c>
+      <c r="D47">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B48" t="str">
+        <v>TG2VernisageLightBlue</v>
+      </c>
+      <c r="C48" t="str">
+        <v/>
+      </c>
+      <c r="D48">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B49" t="str">
+        <v>TG2SymphonyPowder</v>
+      </c>
+      <c r="C49" t="str">
+        <v/>
+      </c>
+      <c r="D49">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B50" t="str">
+        <v>TG2GrungeTurquoise</v>
+      </c>
+      <c r="C50" t="str">
+        <v/>
+      </c>
+      <c r="D50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B51" t="str">
+        <v>TG2VichyDarkBlue</v>
+      </c>
+      <c r="C51" t="str">
+        <v/>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B52" t="str">
+        <v>TG2SymphonyFist</v>
+      </c>
+      <c r="C52" t="str">
+        <v/>
+      </c>
+      <c r="D52">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B53" t="str">
+        <v>TG2FlowersSakuraLavanda</v>
+      </c>
+      <c r="C53" t="str">
+        <v/>
+      </c>
+      <c r="D53">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B54" t="str">
+        <v>TG2ContourBZ</v>
+      </c>
+      <c r="C54" t="str">
+        <v/>
+      </c>
+      <c r="D54">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B55" t="str">
+        <v>TG2ContourLightGrey</v>
+      </c>
+      <c r="C55" t="str">
+        <v/>
+      </c>
+      <c r="D55">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B56" t="str">
+        <v>TG2colibri</v>
+      </c>
+      <c r="C56" t="str">
+        <v/>
+      </c>
+      <c r="D56">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B57" t="str">
+        <v>TG2GraciaGreen</v>
+      </c>
+      <c r="C57" t="str">
+        <v/>
+      </c>
+      <c r="D57">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B58" t="str">
+        <v>TG2CubicGrey</v>
+      </c>
+      <c r="C58" t="str">
+        <v/>
+      </c>
+      <c r="D58">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B59" t="str">
+        <v>TG2WesternOrange</v>
+      </c>
+      <c r="C59" t="str">
+        <v/>
+      </c>
+      <c r="D59">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B60" t="str">
+        <v>TG2BanansGreen</v>
+      </c>
+      <c r="C60" t="str">
+        <v/>
+      </c>
+      <c r="D60">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B61" t="str">
+        <v>TG2EllipsTurquoiseGreen</v>
+      </c>
+      <c r="C61" t="str">
+        <v/>
+      </c>
+      <c r="D61">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B62" t="str">
+        <v>TG2FeeriyaBluePurple</v>
+      </c>
+      <c r="C62" t="str">
+        <v/>
+      </c>
+      <c r="D62">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B63" t="str">
+        <v>TG2Margaritka</v>
+      </c>
+      <c r="C63" t="str">
+        <v/>
+      </c>
+      <c r="D63">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B64" t="str">
+        <v>TG2TropicanaGreyTurquoise</v>
+      </c>
+      <c r="C64" t="str">
+        <v/>
+      </c>
+      <c r="D64">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B65" t="str">
+        <v>TG3DialoguePink220/33</v>
+      </c>
+      <c r="C65" t="str">
+        <v/>
+      </c>
+      <c r="D65">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B66" t="str">
+        <v>TG3ColiseyWhite220/33</v>
+      </c>
+      <c r="C66" t="str">
+        <v/>
+      </c>
+      <c r="D66">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B67" t="str">
+        <v>TG3TotemYellow220/33</v>
+      </c>
+      <c r="C67" t="str">
+        <v/>
+      </c>
+      <c r="D67">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B68" t="str">
+        <v>TG3Lyric220/33</v>
+      </c>
+      <c r="C68" t="str">
+        <v/>
+      </c>
+      <c r="D68">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B69" t="str">
+        <v>TG3SozvezdieBlack220/33</v>
+      </c>
+      <c r="C69" t="str">
+        <v/>
+      </c>
+      <c r="D69">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B70" t="str">
+        <v>TG3PoligonsDeepBlue220/33</v>
+      </c>
+      <c r="C70" t="str">
+        <v/>
+      </c>
+      <c r="D70">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B71" t="str">
+        <v>TG3EucaliptusPink220/33</v>
+      </c>
+      <c r="C71" t="str">
+        <v/>
+      </c>
+      <c r="D71">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B72" t="str">
+        <v>TG3WesternGrey220/33</v>
+      </c>
+      <c r="C72" t="str">
+        <v/>
+      </c>
+      <c r="D72">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B73" t="str">
+        <v>TG3Grani220/33</v>
+      </c>
+      <c r="C73" t="str">
+        <v/>
+      </c>
+      <c r="D73">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B74" t="str">
+        <v>TG3VivienWhiteBlue</v>
+      </c>
+      <c r="C74" t="str">
+        <v/>
+      </c>
+      <c r="D74">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B75" t="str">
+        <v>TG3ConfettiBlue220/33</v>
+      </c>
+      <c r="C75" t="str">
+        <v/>
+      </c>
+      <c r="D75">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B76" t="str">
+        <v>TG3IllusionGrey220/33</v>
+      </c>
+      <c r="C76" t="str">
+        <v/>
+      </c>
+      <c r="D76">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B77" t="str">
+        <v>TG3ConfettiBrown220/33</v>
+      </c>
+      <c r="C77" t="str">
+        <v/>
+      </c>
+      <c r="D77">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B78" t="str">
+        <v>TG3TattersolWhiteEarth220/33</v>
+      </c>
+      <c r="C78" t="str">
+        <v/>
+      </c>
+      <c r="D78">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B79" t="str">
+        <v>TG3RomanticPowdery220/33</v>
+      </c>
+      <c r="C79" t="str">
+        <v/>
+      </c>
+      <c r="D79">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B80" t="str">
+        <v>TG3PapayaBeloZemel220/33</v>
+      </c>
+      <c r="C80" t="str">
+        <v/>
+      </c>
+      <c r="D80">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B81" t="str">
+        <v>TG3ContourBejeviy220/33</v>
+      </c>
+      <c r="C81" t="str">
+        <v/>
+      </c>
+      <c r="D81">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B82" t="str">
+        <v>TG3DialogueTurquoise</v>
+      </c>
+      <c r="C82" t="str">
+        <v/>
+      </c>
+      <c r="D82">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B83" t="str">
+        <v>TG3MagnoliiLavanda</v>
+      </c>
+      <c r="C83" t="str">
+        <v/>
+      </c>
+      <c r="D83">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B84" t="str">
+        <v>TG3TattersolLightGrey</v>
+      </c>
+      <c r="C84" t="str">
+        <v/>
+      </c>
+      <c r="D84">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B85" t="str">
+        <v>TG3ValenciaBZ</v>
+      </c>
+      <c r="C85" t="str">
+        <v/>
+      </c>
+      <c r="D85">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B86" t="str">
+        <v>TG3TattersolLightBlue</v>
+      </c>
+      <c r="C86" t="str">
+        <v/>
+      </c>
+      <c r="D86">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B87" t="str">
+        <v>TG3FleurTurquoise</v>
+      </c>
+      <c r="C87" t="str">
+        <v/>
+      </c>
+      <c r="D87">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B88" t="str">
+        <v>TG3TreugMocco</v>
+      </c>
+      <c r="C88" t="str">
+        <v/>
+      </c>
+      <c r="D88">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B89" t="str">
+        <v>TG3MaroccoLightBlue</v>
+      </c>
+      <c r="C89" t="str">
+        <v/>
+      </c>
+      <c r="D89">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B90" t="str">
+        <v>TG3TattersolSeaWave</v>
+      </c>
+      <c r="C90" t="str">
+        <v/>
+      </c>
+      <c r="D90">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B91" t="str">
+        <v>TG3ValenciaBej</v>
+      </c>
+      <c r="C91" t="str">
+        <v/>
+      </c>
+      <c r="D91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B92" t="str">
+        <v>TG3JungleLightGreen</v>
+      </c>
+      <c r="C92" t="str">
+        <v/>
+      </c>
+      <c r="D92">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B93" t="str">
+        <v>TG3StripePowder</v>
+      </c>
+      <c r="C93" t="str">
+        <v/>
+      </c>
+      <c r="D93">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B94" t="str">
+        <v>TG3StripeSilver</v>
+      </c>
+      <c r="C94" t="str">
+        <v/>
+      </c>
+      <c r="D94">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B95" t="str">
+        <v>TG3FidgieBeidge220/33</v>
+      </c>
+      <c r="C95" t="str">
+        <v/>
+      </c>
+      <c r="D95">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B96" t="str">
+        <v>TG3Raduga</v>
+      </c>
+      <c r="C96" t="str">
+        <v/>
+      </c>
+      <c r="D96">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B97" t="str">
+        <v>LabirintBrown-TG8</v>
+      </c>
+      <c r="C97" t="str">
+        <v/>
+      </c>
+      <c r="D97">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B98" t="str">
+        <v>DunovenieGreyBeige-TG8</v>
+      </c>
+      <c r="C98" t="str">
+        <v/>
+      </c>
+      <c r="D98">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B99" t="str">
+        <v>FidgieBeidge-TG8</v>
+      </c>
+      <c r="C99" t="str">
+        <v/>
+      </c>
+      <c r="D99">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B100" t="str">
+        <v>Banans-TG8</v>
+      </c>
+      <c r="C100" t="str">
+        <v/>
+      </c>
+      <c r="D100">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B101" t="str">
+        <v>CreativeGreyBej-TG8</v>
+      </c>
+      <c r="C101" t="str">
+        <v/>
+      </c>
+      <c r="D101">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B102" t="str">
+        <v>GraciaGreen-TG8</v>
+      </c>
+      <c r="C102" t="str">
+        <v/>
+      </c>
+      <c r="D102">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B103" t="str">
+        <v>FlowersSakurPowder-TG8</v>
+      </c>
+      <c r="C103" t="str">
+        <v/>
+      </c>
+      <c r="D103">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B104" t="str">
+        <v>MargaritkaGreen-TG8</v>
+      </c>
+      <c r="C104" t="str">
+        <v/>
+      </c>
+      <c r="D104">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B105" t="str">
+        <v>EucaliptusBlue-TG8</v>
+      </c>
+      <c r="C105" t="str">
+        <v/>
+      </c>
+      <c r="D105">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B106" t="str">
+        <v>TattersolBZ-TG8</v>
+      </c>
+      <c r="C106" t="str">
+        <v/>
+      </c>
+      <c r="D106">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B107" t="str">
+        <v>ValenciaTurquoiseGreen-TG8</v>
+      </c>
+      <c r="C107" t="str">
+        <v/>
+      </c>
+      <c r="D107">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B108" t="str">
+        <v>ValenciaBZ-TG8</v>
+      </c>
+      <c r="C108" t="str">
+        <v/>
+      </c>
+      <c r="D108">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B109" t="str">
+        <v>LabirintVasilek-TG8</v>
+      </c>
+      <c r="C109" t="str">
+        <v/>
+      </c>
+      <c r="D109">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B110" t="str">
+        <v>LondonTurquoise-TG8</v>
+      </c>
+      <c r="C110" t="str">
+        <v/>
+      </c>
+      <c r="D110">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B111" t="str">
+        <v>StripePowder-TG8</v>
+      </c>
+      <c r="C111" t="str">
+        <v/>
+      </c>
+      <c r="D111">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B112" t="str">
+        <v>DialogueTurquoise-TG8</v>
+      </c>
+      <c r="C112" t="str">
+        <v/>
+      </c>
+      <c r="D112">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B113" t="str">
+        <v>IllusionGrey-TG8</v>
+      </c>
+      <c r="C113" t="str">
+        <v/>
+      </c>
+      <c r="D113">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B114" t="str">
+        <v>Ellips-TG8</v>
+      </c>
+      <c r="C114" t="str">
+        <v/>
+      </c>
+      <c r="D114">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B115" t="str">
+        <v>ConfettiViolet-TG8</v>
+      </c>
+      <c r="C115" t="str">
+        <v/>
+      </c>
+      <c r="D115">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B116" t="str">
+        <v>ValenciaBlueLiliac-TG8</v>
+      </c>
+      <c r="C116" t="str">
+        <v/>
+      </c>
+      <c r="D116">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B117" t="str">
+        <v>StripeSilver-TG8</v>
+      </c>
+      <c r="C117" t="str">
+        <v/>
+      </c>
+      <c r="D117">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B118" t="str">
+        <v>TattersolLightGrey-TG8</v>
+      </c>
+      <c r="C118" t="str">
+        <v/>
+      </c>
+      <c r="D118">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B119" t="str">
+        <v>FleurTurquoise-TG8</v>
+      </c>
+      <c r="C119" t="str">
+        <v/>
+      </c>
+      <c r="D119">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B120" t="str">
+        <v>EucaliptusPink-TG8</v>
+      </c>
+      <c r="C120" t="str">
+        <v/>
+      </c>
+      <c r="D120">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B121" t="str">
+        <v>MramorGrey-TG8</v>
+      </c>
+      <c r="C121" t="str">
+        <v/>
+      </c>
+      <c r="D121">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B122" t="str">
+        <v>CubicGrey-TG8</v>
+      </c>
+      <c r="C122" t="str">
+        <v/>
+      </c>
+      <c r="D122">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B123" t="str">
+        <v>FeeriyaBluePurple-TG8</v>
+      </c>
+      <c r="C123" t="str">
+        <v/>
+      </c>
+      <c r="D123">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B124" t="str">
+        <v>WesternOrange-TG8</v>
+      </c>
+      <c r="C124" t="str">
+        <v/>
+      </c>
+      <c r="D124">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B125" t="str">
+        <v>TropicanaBej-TG8</v>
+      </c>
+      <c r="C125" t="str">
+        <v/>
+      </c>
+      <c r="D125">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B126" t="str">
+        <v>TropicanaGreyTurquoise-TG8</v>
+      </c>
+      <c r="C126" t="str">
+        <v/>
+      </c>
+      <c r="D126">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B127" t="str">
+        <v>MonblanColour-TG8</v>
+      </c>
+      <c r="C127" t="str">
+        <v/>
+      </c>
+      <c r="D127">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B128" t="str">
+        <v>Raduga-TG8</v>
+      </c>
+      <c r="C128" t="str">
+        <v/>
+      </c>
+      <c r="D128">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B129" t="str">
+        <v>KaramelBZ-TG8</v>
+      </c>
+      <c r="C129" t="str">
+        <v/>
+      </c>
+      <c r="D129">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B130" t="str">
+        <v>TattersolGreyBeige-TG8</v>
+      </c>
+      <c r="C130" t="str">
+        <v/>
+      </c>
+      <c r="D130">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B131" t="str">
+        <v>PoligonsDeepBlue-TG8</v>
+      </c>
+      <c r="C131" t="str">
+        <v/>
+      </c>
+      <c r="D131">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B132" t="str">
+        <v>TotemYellow-TG8</v>
+      </c>
+      <c r="C132" t="str">
+        <v/>
+      </c>
+      <c r="D132">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B133" t="str">
+        <v>ContourBZ-TG8</v>
+      </c>
+      <c r="C133" t="str">
+        <v/>
+      </c>
+      <c r="D133">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B134" t="str">
+        <v>CubicBej-TG8</v>
+      </c>
+      <c r="C134" t="str">
+        <v/>
+      </c>
+      <c r="D134">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B135" t="str">
+        <v>RomanticLightBlue-TG8</v>
+      </c>
+      <c r="C135" t="str">
+        <v/>
+      </c>
+      <c r="D135">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B136" t="str">
+        <v>ConfettiBrown-TG8</v>
+      </c>
+      <c r="C136" t="str">
+        <v/>
+      </c>
+      <c r="D136">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B137" t="str">
+        <v>TropicanaBlack-TG8</v>
+      </c>
+      <c r="C137" t="str">
+        <v/>
+      </c>
+      <c r="D137">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B138" t="str">
+        <v>Madlen-TG8</v>
+      </c>
+      <c r="C138" t="str">
+        <v/>
+      </c>
+      <c r="D138">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B139" t="str">
+        <v>RomanticBlue-TG8</v>
+      </c>
+      <c r="C139" t="str">
+        <v/>
+      </c>
+      <c r="D139">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B140" t="str">
+        <v>MramorTurquoise-TG8</v>
+      </c>
+      <c r="C140" t="str">
+        <v/>
+      </c>
+      <c r="D140">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B141" t="str">
+        <v>SymphonyFist-TG8</v>
+      </c>
+      <c r="C141" t="str">
+        <v/>
+      </c>
+      <c r="D141">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B142" t="str">
+        <v>SmilesBZ-TG8</v>
+      </c>
+      <c r="C142" t="str">
+        <v/>
+      </c>
+      <c r="D142">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B143" t="str">
+        <v>TG3ViolettaLavand</v>
+      </c>
+      <c r="C143" t="str">
+        <v/>
+      </c>
+      <c r="D143">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B144" t="str">
+        <v>TG3AmazonkaBZ</v>
+      </c>
+      <c r="C144" t="str">
+        <v/>
+      </c>
+      <c r="D144">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B145" t="str">
+        <v>TG3AmourBeloZemel</v>
+      </c>
+      <c r="C145" t="str">
+        <v/>
+      </c>
+      <c r="D145">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B146" t="str">
+        <v>TG3MagicBordo</v>
+      </c>
+      <c r="C146" t="str">
+        <v/>
+      </c>
+      <c r="D146">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B147" t="str">
+        <v>TG3RadugaBej</v>
+      </c>
+      <c r="C147" t="str">
+        <v/>
+      </c>
+      <c r="D147">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B148" t="str">
+        <v>TG3TucansGreen</v>
+      </c>
+      <c r="C148" t="str">
+        <v/>
+      </c>
+      <c r="D148">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B149" t="str">
+        <v>ViolettaLavand-TG8</v>
+      </c>
+      <c r="C149" t="str">
+        <v/>
+      </c>
+      <c r="D149">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B150" t="str">
+        <v>AmazonkaBZ-TG8</v>
+      </c>
+      <c r="C150" t="str">
+        <v/>
+      </c>
+      <c r="D150">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B151" t="str">
+        <v>AmourBZ-TG8</v>
+      </c>
+      <c r="C151" t="str">
+        <v/>
+      </c>
+      <c r="D151">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B152" t="str">
+        <v>MagicBordo-TG8</v>
+      </c>
+      <c r="C152" t="str">
+        <v/>
+      </c>
+      <c r="D152">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B153" t="str">
+        <v>RadugaBej-TG8</v>
+      </c>
+      <c r="C153" t="str">
+        <v/>
+      </c>
+      <c r="D153">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B154" t="str">
+        <v>TucansGreen-TG8</v>
+      </c>
+      <c r="C154" t="str">
+        <v/>
+      </c>
+      <c r="D154">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B155" t="str">
+        <v>TG3PositiveLightGrey</v>
+      </c>
+      <c r="C155" t="str">
+        <v/>
+      </c>
+      <c r="D155">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B156" t="str">
+        <v>TG3GlorisGrey</v>
+      </c>
+      <c r="C156" t="str">
+        <v/>
+      </c>
+      <c r="D156">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B157" t="str">
+        <v>TG3LetniySadBZ</v>
+      </c>
+      <c r="C157" t="str">
+        <v/>
+      </c>
+      <c r="D157">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B158" t="str">
+        <v>TG3BestFriendBej</v>
+      </c>
+      <c r="C158" t="str">
+        <v/>
+      </c>
+      <c r="D158">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B159" t="str">
+        <v>TG3Jaklin</v>
+      </c>
+      <c r="C159" t="str">
+        <v/>
+      </c>
+      <c r="D159">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B160" t="str">
+        <v>TG3LazurBZLightBlue</v>
+      </c>
+      <c r="C160" t="str">
+        <v/>
+      </c>
+      <c r="D160">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B161" t="str">
+        <v>TG2VizantBejPink33</v>
+      </c>
+      <c r="C161" t="str">
+        <v/>
+      </c>
+      <c r="D161">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B162" t="str">
+        <v>TG2GalaxyChoko33</v>
+      </c>
+      <c r="C162" t="str">
+        <v/>
+      </c>
+      <c r="D162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B163" t="str">
+        <v>TG2JungleTurqGreen33</v>
+      </c>
+      <c r="C163" t="str">
+        <v/>
+      </c>
+      <c r="D163">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B164" t="str">
+        <v>TG2ListopadBZgrey33</v>
+      </c>
+      <c r="C164" t="str">
+        <v/>
+      </c>
+      <c r="D164">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B165" t="str">
+        <v>TG2MilflerBZlightBlue33</v>
+      </c>
+      <c r="C165" t="str">
+        <v/>
+      </c>
+      <c r="D165">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B166" t="str">
+        <v>TG2MilflerBZpink33</v>
+      </c>
+      <c r="C166" t="str">
+        <v/>
+      </c>
+      <c r="D166">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B167" t="str">
+        <v>TG2TartanBZpink33</v>
+      </c>
+      <c r="C167" t="str">
+        <v/>
+      </c>
+      <c r="D167">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B168" t="str">
+        <v>TG2TeoremaGrey33</v>
+      </c>
+      <c r="C168" t="str">
+        <v/>
+      </c>
+      <c r="D168">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B169" t="str">
+        <v>VizantBejPink-TG8</v>
+      </c>
+      <c r="C169" t="str">
+        <v/>
+      </c>
+      <c r="D169">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B170" t="str">
+        <v>GalaxyChoko-TG8</v>
+      </c>
+      <c r="C170" t="str">
+        <v/>
+      </c>
+      <c r="D170">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B171" t="str">
+        <v>JungleTurqGreen-TG8</v>
+      </c>
+      <c r="C171" t="str">
+        <v/>
+      </c>
+      <c r="D171">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B172" t="str">
+        <v>ListopadBZgrey-TG8</v>
+      </c>
+      <c r="C172" t="str">
+        <v/>
+      </c>
+      <c r="D172">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B173" t="str">
+        <v>MilflerBZlightBlue-TG8</v>
+      </c>
+      <c r="C173" t="str">
+        <v/>
+      </c>
+      <c r="D173">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B174" t="str">
+        <v>MilflerBZpink-TG8</v>
+      </c>
+      <c r="C174" t="str">
+        <v/>
+      </c>
+      <c r="D174">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B175" t="str">
+        <v>TartanBZpink-TG8</v>
+      </c>
+      <c r="C175" t="str">
+        <v/>
+      </c>
+      <c r="D175">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B176" t="str">
+        <v>TeoremaGrey-TG8</v>
+      </c>
+      <c r="C176" t="str">
+        <v/>
+      </c>
+      <c r="D176">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B177" t="str">
+        <v>TG2CubicBordo</v>
+      </c>
+      <c r="C177" t="str">
+        <v/>
+      </c>
+      <c r="D177">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B178" t="str">
+        <v>CubicBordo-TG8</v>
+      </c>
+      <c r="C178" t="str">
+        <v/>
+      </c>
+      <c r="D178">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B179" t="str">
+        <v>TG1AvangardBZgrey</v>
+      </c>
+      <c r="C179" t="str">
+        <v/>
+      </c>
+      <c r="D179">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B180" t="str">
+        <v>TG1TatterlineBej</v>
+      </c>
+      <c r="C180" t="str">
+        <v/>
+      </c>
+      <c r="D180">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B181" t="str">
+        <v>TG1TheoremaBej</v>
+      </c>
+      <c r="C181" t="str">
+        <v/>
+      </c>
+      <c r="D181">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B182" t="str">
+        <v>TG1UrbanDarkGrey</v>
+      </c>
+      <c r="C182" t="str">
+        <v/>
+      </c>
+      <c r="D182">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B183" t="str">
+        <v>TatterlineBej-TG8</v>
+      </c>
+      <c r="C183" t="str">
+        <v/>
+      </c>
+      <c r="D183">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B184" t="str">
+        <v>UrbanDarkGrey-TG8</v>
+      </c>
+      <c r="C184" t="str">
+        <v/>
+      </c>
+      <c r="D184">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B185" t="str">
+        <v>AvangardBZgrey-TG8</v>
+      </c>
+      <c r="C185" t="str">
+        <v/>
+      </c>
+      <c r="D185">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B186" t="str">
+        <v>TheoremaBej-TG8</v>
+      </c>
+      <c r="C186" t="str">
+        <v/>
+      </c>
+      <c r="D186">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D186"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fixed bags, changes in GT and LB stocks
</commit_message>
<xml_diff>
--- a/data/ready_stocks/galtex-ozon-stocks-updated.xlsx
+++ b/data/ready_stocks/galtex-ozon-stocks-updated.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D198"/>
+  <dimension ref="A1:D153"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -418,7 +418,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B2" t="str">
-        <v>TG1TropicanaBeige220/33</v>
+        <v>TG5CircusWhiteEarth150/50</v>
       </c>
       <c r="C2" t="str">
         <v/>
@@ -432,13 +432,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B3" t="str">
-        <v>TG1LondonTurquoise220/33</v>
+        <v>TG5losang150/50</v>
       </c>
       <c r="C3" t="str">
         <v/>
       </c>
       <c r="D3">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -446,7 +446,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B4" t="str">
-        <v>TG1MramorTurquoise</v>
+        <v>TG5GraphicOrange150/50</v>
       </c>
       <c r="C4" t="str">
         <v/>
@@ -460,13 +460,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B5" t="str">
-        <v>TG1MramorGrey</v>
+        <v>TG5EucaliptPink150/50</v>
       </c>
       <c r="C5" t="str">
         <v/>
       </c>
       <c r="D5">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -474,7 +474,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B6" t="str">
-        <v>TG1ValenciaBlueLiliac</v>
+        <v>TG5stripeViol150/50</v>
       </c>
       <c r="C6" t="str">
         <v/>
@@ -488,7 +488,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B7" t="str">
-        <v>TG1MonblanColour</v>
+        <v>TG5CatHomeDeepBlue150/50</v>
       </c>
       <c r="C7" t="str">
         <v/>
@@ -502,7 +502,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B8" t="str">
-        <v>TG1VoskhodOrange</v>
+        <v>TG5FlowerSakurLavand150/50</v>
       </c>
       <c r="C8" t="str">
         <v/>
@@ -516,7 +516,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B9" t="str">
-        <v>TG1KaramelBZ</v>
+        <v>TG5kotbaton150/50</v>
       </c>
       <c r="C9" t="str">
         <v/>
@@ -530,13 +530,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B10" t="str">
-        <v>TG1VichyBej</v>
+        <v>TG5BibigonBej150/50</v>
       </c>
       <c r="C10" t="str">
         <v/>
       </c>
       <c r="D10">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -544,7 +544,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B11" t="str">
-        <v>TG1RomanticBlue</v>
+        <v>TG5GraphicChoco150/50</v>
       </c>
       <c r="C11" t="str">
         <v/>
@@ -558,7 +558,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B12" t="str">
-        <v>TG1SymphonyGreyBej</v>
+        <v>TG5CatHomeDeepGrey150/50</v>
       </c>
       <c r="C12" t="str">
         <v/>
@@ -572,13 +572,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B13" t="str">
-        <v>TG1ValenciaTurquoiseGreen</v>
+        <v>TG5gta150/50</v>
       </c>
       <c r="C13" t="str">
         <v/>
       </c>
       <c r="D13">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14">
@@ -586,7 +586,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B14" t="str">
-        <v>TG1TropicTurquoise</v>
+        <v>TG5stripeChoco150/50</v>
       </c>
       <c r="C14" t="str">
         <v/>
@@ -600,13 +600,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B15" t="str">
-        <v>TG1TropicanaBlack</v>
+        <v>TG5EucaliptBlue150/50</v>
       </c>
       <c r="C15" t="str">
         <v/>
       </c>
       <c r="D15">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -614,13 +614,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B16" t="str">
-        <v>TG1TattersolGreyBej</v>
+        <v>TG5Grani</v>
       </c>
       <c r="C16" t="str">
         <v/>
       </c>
       <c r="D16">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -628,7 +628,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B17" t="str">
-        <v>TG1TreugLightBlue220/33</v>
+        <v>TG5TreugolnikiTurquoise</v>
       </c>
       <c r="C17" t="str">
         <v/>
@@ -642,13 +642,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B18" t="str">
-        <v>TG1NiagaraTurquoise</v>
+        <v>TG5TattersolBZ</v>
       </c>
       <c r="C18" t="str">
         <v/>
       </c>
       <c r="D18">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -656,7 +656,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B19" t="str">
-        <v>TG1NiagaraYellow</v>
+        <v>TG5SymphonyPowder</v>
       </c>
       <c r="C19" t="str">
         <v/>
@@ -670,7 +670,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B20" t="str">
-        <v>TG1Smiles</v>
+        <v>TG5HollywoodDarkBeige</v>
       </c>
       <c r="C20" t="str">
         <v/>
@@ -684,13 +684,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B21" t="str">
-        <v>TG1Aquarelle</v>
+        <v>TG5animeDarkGrey</v>
       </c>
       <c r="C21" t="str">
         <v/>
       </c>
       <c r="D21">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -698,13 +698,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B22" t="str">
-        <v>TG1BogemaTurquoise</v>
+        <v>TG5FlyBZ</v>
       </c>
       <c r="C22" t="str">
         <v/>
       </c>
       <c r="D22">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -712,7 +712,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B23" t="str">
-        <v>TG1MadlenGrey</v>
+        <v>TG5BeskonechnostBZ</v>
       </c>
       <c r="C23" t="str">
         <v/>
@@ -726,7 +726,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B24" t="str">
-        <v>TG1ZavitokChoco</v>
+        <v>TG5ZavitokLavanda</v>
       </c>
       <c r="C24" t="str">
         <v/>
@@ -740,13 +740,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B25" t="str">
-        <v>TG1CubicBej</v>
+        <v>TG5KletochkaTurquoise</v>
       </c>
       <c r="C25" t="str">
         <v/>
       </c>
       <c r="D25">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -754,7 +754,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B26" t="str">
-        <v>TG1RomanticLightBlue</v>
+        <v>TG5StrekoziGreyBeige</v>
       </c>
       <c r="C26" t="str">
         <v/>
@@ -768,7 +768,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B27" t="str">
-        <v>TG1ConfettiLime</v>
+        <v>TG5VichyLightBlue</v>
       </c>
       <c r="C27" t="str">
         <v/>
@@ -782,7 +782,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B28" t="str">
-        <v>TG1Florans</v>
+        <v>TG5GlorisGrey</v>
       </c>
       <c r="C28" t="str">
         <v/>
@@ -796,13 +796,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B29" t="str">
-        <v>TG1BeskonechnostBZ</v>
+        <v>TG5LabirintBrown</v>
       </c>
       <c r="C29" t="str">
         <v/>
       </c>
       <c r="D29">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="30">
@@ -810,13 +810,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B30" t="str">
-        <v>TG1JungleGreyBej</v>
+        <v>TG5SymphonyLightBlue</v>
       </c>
       <c r="C30" t="str">
         <v/>
       </c>
       <c r="D30">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -824,13 +824,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B31" t="str">
-        <v>TG1BogemaGrey</v>
+        <v>TG5ContourBeige</v>
       </c>
       <c r="C31" t="str">
         <v/>
       </c>
       <c r="D31">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -838,7 +838,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B32" t="str">
-        <v>TG1GraciaBZgrey</v>
+        <v>TG5TropicTurquoise</v>
       </c>
       <c r="C32" t="str">
         <v/>
@@ -852,13 +852,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B33" t="str">
-        <v>TG2EucaliptusBlue220/33</v>
+        <v>TG5SladkieSniGrafit</v>
       </c>
       <c r="C33" t="str">
         <v/>
       </c>
       <c r="D33">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -866,7 +866,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B34" t="str">
-        <v>TG2WesternSeaWave220/33</v>
+        <v>TG5ShtrikhiMocco</v>
       </c>
       <c r="C34" t="str">
         <v/>
@@ -880,7 +880,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B35" t="str">
-        <v>TG2SonetBZ</v>
+        <v>TG5BibigonGreen</v>
       </c>
       <c r="C35" t="str">
         <v/>
@@ -894,7 +894,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B36" t="str">
-        <v>TG2FlowersSakurPowder</v>
+        <v>TG5TropicanaGreyTurquoise</v>
       </c>
       <c r="C36" t="str">
         <v/>
@@ -908,7 +908,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B37" t="str">
-        <v>TG2DunovenieGreyBeige</v>
+        <v>TG5ZavitokLightBlue</v>
       </c>
       <c r="C37" t="str">
         <v/>
@@ -922,7 +922,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B38" t="str">
-        <v>TG2ContourGreen</v>
+        <v>TG5PandaBeige</v>
       </c>
       <c r="C38" t="str">
         <v/>
@@ -936,13 +936,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B39" t="str">
-        <v>TG2LabirintBrown</v>
+        <v>TG5QuestBZGreen</v>
       </c>
       <c r="C39" t="str">
         <v/>
       </c>
       <c r="D39">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="40">
@@ -950,13 +950,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B40" t="str">
-        <v>TG2WesternPowder</v>
+        <v>TG5BogemaTurquoise</v>
       </c>
       <c r="C40" t="str">
         <v/>
       </c>
       <c r="D40">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="41">
@@ -964,13 +964,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B41" t="str">
-        <v>TG2EverestDarkGrey</v>
+        <v>TG5StepBlack</v>
       </c>
       <c r="C41" t="str">
         <v/>
       </c>
       <c r="D41">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
@@ -978,13 +978,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B42" t="str">
-        <v>TG2CreativeGreyBej</v>
+        <v>TG5RozaPink</v>
       </c>
       <c r="C42" t="str">
         <v/>
       </c>
       <c r="D42">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -992,13 +992,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B43" t="str">
-        <v>TG2ContourDarkGrey</v>
+        <v>TG5StripePowder</v>
       </c>
       <c r="C43" t="str">
         <v/>
       </c>
       <c r="D43">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -1006,13 +1006,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B44" t="str">
-        <v>TG2CollageBejBlue</v>
+        <v>TG5StrekoziMint</v>
       </c>
       <c r="C44" t="str">
         <v/>
       </c>
       <c r="D44">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="45">
@@ -1020,7 +1020,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B45" t="str">
-        <v>TG2SymphonyLightBlue</v>
+        <v>TG5TropicanaBej</v>
       </c>
       <c r="C45" t="str">
         <v/>
@@ -1034,13 +1034,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B46" t="str">
-        <v>TG2VernisageLightBlue</v>
+        <v>TG5GoodNightLightBlue</v>
       </c>
       <c r="C46" t="str">
         <v/>
       </c>
       <c r="D46">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -1048,7 +1048,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B47" t="str">
-        <v>TG2SymphonyPowder</v>
+        <v>TG5MishkiWhiteGreen</v>
       </c>
       <c r="C47" t="str">
         <v/>
@@ -1062,7 +1062,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B48" t="str">
-        <v>TG2GrungeTurquoise</v>
+        <v>TG5DialoguePink</v>
       </c>
       <c r="C48" t="str">
         <v/>
@@ -1076,13 +1076,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B49" t="str">
-        <v>TG2VichyDarkBlue</v>
+        <v>TG5PolosatieMishkiBZ</v>
       </c>
       <c r="C49" t="str">
         <v/>
       </c>
       <c r="D49">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="50">
@@ -1090,13 +1090,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B50" t="str">
-        <v>TG2SymphonyFist</v>
+        <v>TG5StarNightBlack</v>
       </c>
       <c r="C50" t="str">
         <v/>
       </c>
       <c r="D50">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="51">
@@ -1104,7 +1104,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B51" t="str">
-        <v>TG2FlowersSakuraLavanda</v>
+        <v>TG5Kotovasia</v>
       </c>
       <c r="C51" t="str">
         <v/>
@@ -1118,7 +1118,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B52" t="str">
-        <v>TG2ContourBZ</v>
+        <v>TG5StripeSilver</v>
       </c>
       <c r="C52" t="str">
         <v/>
@@ -1132,7 +1132,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B53" t="str">
-        <v>TG2ContourLightGrey</v>
+        <v>TG5ZaikiWhiteBlue</v>
       </c>
       <c r="C53" t="str">
         <v/>
@@ -1146,13 +1146,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B54" t="str">
-        <v>TG2colibri</v>
+        <v>TG5KletochkaMint</v>
       </c>
       <c r="C54" t="str">
         <v/>
       </c>
       <c r="D54">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="55">
@@ -1160,7 +1160,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B55" t="str">
-        <v>TG2GraciaGreen</v>
+        <v>TG5MramorTurquoise</v>
       </c>
       <c r="C55" t="str">
         <v/>
@@ -1174,13 +1174,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B56" t="str">
-        <v>TG2CubicGrey</v>
+        <v>TG5ArabeskiLightBlue</v>
       </c>
       <c r="C56" t="str">
         <v/>
       </c>
       <c r="D56">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57">
@@ -1188,13 +1188,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B57" t="str">
-        <v>TG2WesternOrange</v>
+        <v>TG5MishkiWhiteYellow</v>
       </c>
       <c r="C57" t="str">
         <v/>
       </c>
       <c r="D57">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58">
@@ -1202,13 +1202,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B58" t="str">
-        <v>TG2BanansGreen</v>
+        <v>TG5GooseOtosplus</v>
       </c>
       <c r="C58" t="str">
         <v/>
       </c>
       <c r="D58">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59">
@@ -1216,13 +1216,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B59" t="str">
-        <v>TG2EllipsTurquoiseGreen</v>
+        <v>TG5DialogueTurquoise</v>
       </c>
       <c r="C59" t="str">
         <v/>
       </c>
       <c r="D59">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60">
@@ -1230,7 +1230,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B60" t="str">
-        <v>TG2FeeriyaBluePurple</v>
+        <v>TG5Florans</v>
       </c>
       <c r="C60" t="str">
         <v/>
@@ -1244,13 +1244,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B61" t="str">
-        <v>TG2Margaritka</v>
+        <v>TG5ZavitokChoco</v>
       </c>
       <c r="C61" t="str">
         <v/>
       </c>
       <c r="D61">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62">
@@ -1258,7 +1258,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B62" t="str">
-        <v>TG2TropicanaGreyTurquoise</v>
+        <v>TG5BanansGreen</v>
       </c>
       <c r="C62" t="str">
         <v/>
@@ -1272,13 +1272,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B63" t="str">
-        <v>TG3DialoguePink220/33</v>
+        <v>TG5SmilesGrey</v>
       </c>
       <c r="C63" t="str">
         <v/>
       </c>
       <c r="D63">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64">
@@ -1286,7 +1286,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B64" t="str">
-        <v>TG3ColiseyWhite220/33</v>
+        <v>TG5StrekoziLightBlue</v>
       </c>
       <c r="C64" t="str">
         <v/>
@@ -1300,13 +1300,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B65" t="str">
-        <v>TG3TotemYellow220/33</v>
+        <v>TG5MishkiWhiteBlue</v>
       </c>
       <c r="C65" t="str">
         <v/>
       </c>
       <c r="D65">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66">
@@ -1314,13 +1314,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B66" t="str">
-        <v>TG3Lyric220/33</v>
+        <v>TG5ValenciaBlueLiliac</v>
       </c>
       <c r="C66" t="str">
         <v/>
       </c>
       <c r="D66">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="67">
@@ -1328,7 +1328,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B67" t="str">
-        <v>TG3SozvezdieBlack220/33</v>
+        <v>TG5LondonTurquoise</v>
       </c>
       <c r="C67" t="str">
         <v/>
@@ -1342,13 +1342,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B68" t="str">
-        <v>TG3PoligonsDeepBlue220/33</v>
+        <v>TG5TropicanaBlack</v>
       </c>
       <c r="C68" t="str">
         <v/>
       </c>
       <c r="D68">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="69">
@@ -1356,13 +1356,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B69" t="str">
-        <v>TG3EucaliptusPink220/33</v>
+        <v>TG5WesternPowder</v>
       </c>
       <c r="C69" t="str">
         <v/>
       </c>
       <c r="D69">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="70">
@@ -1370,13 +1370,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B70" t="str">
-        <v>TG3WesternGrey220/33</v>
+        <v>TG5ValenciaGreenTurq</v>
       </c>
       <c r="C70" t="str">
         <v/>
       </c>
       <c r="D70">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71">
@@ -1384,7 +1384,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B71" t="str">
-        <v>TG3Grani220/33</v>
+        <v>TG5ZooparkGreen</v>
       </c>
       <c r="C71" t="str">
         <v/>
@@ -1398,7 +1398,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B72" t="str">
-        <v>TG3VivienWhiteBlue</v>
+        <v>TG5VenzelBej</v>
       </c>
       <c r="C72" t="str">
         <v/>
@@ -1412,13 +1412,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B73" t="str">
-        <v>TG3ConfettiBlue220/33</v>
+        <v>TG5ValenciaBej</v>
       </c>
       <c r="C73" t="str">
         <v/>
       </c>
       <c r="D73">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74">
@@ -1426,7 +1426,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B74" t="str">
-        <v>TG3IllusionGrey220/33</v>
+        <v>TG5ValenciaBZ</v>
       </c>
       <c r="C74" t="str">
         <v/>
@@ -1440,13 +1440,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B75" t="str">
-        <v>TG3ConfettiBrown220/33</v>
+        <v>TG5TattersolGreyBej</v>
       </c>
       <c r="C75" t="str">
         <v/>
       </c>
       <c r="D75">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="76">
@@ -1454,13 +1454,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B76" t="str">
-        <v>TG3TattersolWhiteEarth220/33</v>
+        <v>TG5StarLightGrey</v>
       </c>
       <c r="C76" t="str">
         <v/>
       </c>
       <c r="D76">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="77">
@@ -1468,7 +1468,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B77" t="str">
-        <v>TG3RomanticPowdery220/33</v>
+        <v>TG5StarTurquoise</v>
       </c>
       <c r="C77" t="str">
         <v/>
@@ -1482,7 +1482,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B78" t="str">
-        <v>TG3PapayaBeloZemel220/33</v>
+        <v>TG5GTAColor</v>
       </c>
       <c r="C78" t="str">
         <v/>
@@ -1496,13 +1496,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B79" t="str">
-        <v>TG3ContourBejeviy220/33</v>
+        <v>TG5PerfectNiagara</v>
       </c>
       <c r="C79" t="str">
         <v/>
       </c>
       <c r="D79">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="80">
@@ -1510,7 +1510,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B80" t="str">
-        <v>TG3DialogueTurquoise</v>
+        <v>TG5IllusionGrey</v>
       </c>
       <c r="C80" t="str">
         <v/>
@@ -1524,7 +1524,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B81" t="str">
-        <v>TG3MagnoliiLavanda</v>
+        <v>TG5LabirintVasilek</v>
       </c>
       <c r="C81" t="str">
         <v/>
@@ -1538,7 +1538,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B82" t="str">
-        <v>TG3TattersolLightGrey</v>
+        <v>TG5ContourLightGrey</v>
       </c>
       <c r="C82" t="str">
         <v/>
@@ -1552,7 +1552,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B83" t="str">
-        <v>TG3ValenciaBZ</v>
+        <v>TG5Colibri</v>
       </c>
       <c r="C83" t="str">
         <v/>
@@ -1566,13 +1566,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B84" t="str">
-        <v>TG3TattersolLightBlue</v>
+        <v>TG5SmilesBZWhite</v>
       </c>
       <c r="C84" t="str">
         <v/>
       </c>
       <c r="D84">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85">
@@ -1580,7 +1580,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B85" t="str">
-        <v>TG3FleurTurquoise</v>
+        <v>TG5PoligonSeaWave</v>
       </c>
       <c r="C85" t="str">
         <v/>
@@ -1594,7 +1594,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B86" t="str">
-        <v>TG3TreugMocco</v>
+        <v>TG5LetniySad</v>
       </c>
       <c r="C86" t="str">
         <v/>
@@ -1608,7 +1608,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B87" t="str">
-        <v>TG3MaroccoLightBlue</v>
+        <v>TG5KletochkaBej</v>
       </c>
       <c r="C87" t="str">
         <v/>
@@ -1622,7 +1622,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B88" t="str">
-        <v>TG3TattersolSeaWave</v>
+        <v>TG5Creative</v>
       </c>
       <c r="C88" t="str">
         <v/>
@@ -1636,13 +1636,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B89" t="str">
-        <v>TG3ValenciaBej</v>
+        <v>TG5SozvezdieBlack</v>
       </c>
       <c r="C89" t="str">
         <v/>
       </c>
       <c r="D89">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="90">
@@ -1650,13 +1650,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B90" t="str">
-        <v>TG3JungleLightGreen</v>
+        <v>TG5OwlHomeBejPink</v>
       </c>
       <c r="C90" t="str">
         <v/>
       </c>
       <c r="D90">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="91">
@@ -1664,7 +1664,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B91" t="str">
-        <v>TG3StripePowder</v>
+        <v>TG5FloransBZsiren</v>
       </c>
       <c r="C91" t="str">
         <v/>
@@ -1678,7 +1678,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B92" t="str">
-        <v>TG3StripeSilver</v>
+        <v>TG5BestFriendBej</v>
       </c>
       <c r="C92" t="str">
         <v/>
@@ -1692,7 +1692,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B93" t="str">
-        <v>TG3FidgieBeidge220/33</v>
+        <v>TG5Lyric</v>
       </c>
       <c r="C93" t="str">
         <v/>
@@ -1706,13 +1706,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B94" t="str">
-        <v>TG3Raduga</v>
+        <v>TG5FlowersSakuraPowder</v>
       </c>
       <c r="C94" t="str">
         <v/>
       </c>
       <c r="D94">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="95">
@@ -1720,7 +1720,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B95" t="str">
-        <v>LabirintBrown-TG8</v>
+        <v>TG5CapyBej</v>
       </c>
       <c r="C95" t="str">
         <v/>
@@ -1734,13 +1734,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B96" t="str">
-        <v>DunovenieGreyBeige-TG8</v>
+        <v>TG5GraciaIzumrud</v>
       </c>
       <c r="C96" t="str">
         <v/>
       </c>
       <c r="D96">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="97">
@@ -1748,13 +1748,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B97" t="str">
-        <v>FidgieBeidge-TG8</v>
+        <v>TG5GalaxyChok50</v>
       </c>
       <c r="C97" t="str">
         <v/>
       </c>
       <c r="D97">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="98">
@@ -1762,13 +1762,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B98" t="str">
-        <v>Banans-TG8</v>
+        <v>TG5AmourBZ</v>
       </c>
       <c r="C98" t="str">
         <v/>
       </c>
       <c r="D98">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="99">
@@ -1776,7 +1776,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B99" t="str">
-        <v>CreativeGreyBej-TG8</v>
+        <v>TG5BogemaGrey</v>
       </c>
       <c r="C99" t="str">
         <v/>
@@ -1790,7 +1790,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B100" t="str">
-        <v>GraciaGreen-TG8</v>
+        <v>TG5ContourDarkGrey</v>
       </c>
       <c r="C100" t="str">
         <v/>
@@ -1804,7 +1804,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B101" t="str">
-        <v>FlowersSakurPowder-TG8</v>
+        <v>TG5Fidgie</v>
       </c>
       <c r="C101" t="str">
         <v/>
@@ -1818,13 +1818,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B102" t="str">
-        <v>MargaritkaGreen-TG8</v>
+        <v>TG5GraciaBZgrey</v>
       </c>
       <c r="C102" t="str">
         <v/>
       </c>
       <c r="D102">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="103">
@@ -1832,13 +1832,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B103" t="str">
-        <v>EucaliptusBlue-TG8</v>
+        <v>TG5HollywoodBlue</v>
       </c>
       <c r="C103" t="str">
         <v/>
       </c>
       <c r="D103">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="104">
@@ -1846,7 +1846,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B104" t="str">
-        <v>TattersolBZ-TG8</v>
+        <v>TG5KotAkula</v>
       </c>
       <c r="C104" t="str">
         <v/>
@@ -1860,7 +1860,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B105" t="str">
-        <v>ValenciaTurquoiseGreen-TG8</v>
+        <v>TG5LavandBuketBZ</v>
       </c>
       <c r="C105" t="str">
         <v/>
@@ -1874,7 +1874,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B106" t="str">
-        <v>ValenciaBZ-TG8</v>
+        <v>TG5MilflerBZpink</v>
       </c>
       <c r="C106" t="str">
         <v/>
@@ -1888,13 +1888,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B107" t="str">
-        <v>LabirintVasilek-TG8</v>
+        <v>TG5SymphGreyBej</v>
       </c>
       <c r="C107" t="str">
         <v/>
       </c>
       <c r="D107">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="108">
@@ -1902,13 +1902,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B108" t="str">
-        <v>LondonTurquoise-TG8</v>
+        <v>TG5TartanBZgrey</v>
       </c>
       <c r="C108" t="str">
         <v/>
       </c>
       <c r="D108">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="109">
@@ -1916,7 +1916,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B109" t="str">
-        <v>StripePowder-TG8</v>
+        <v>TG5TheoremBej</v>
       </c>
       <c r="C109" t="str">
         <v/>
@@ -1930,13 +1930,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B110" t="str">
-        <v>DialogueTurquoise-TG8</v>
+        <v>TG5TheoremGrey</v>
       </c>
       <c r="C110" t="str">
         <v/>
       </c>
       <c r="D110">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="111">
@@ -1944,7 +1944,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B111" t="str">
-        <v>IllusionGrey-TG8</v>
+        <v>TG5Totem</v>
       </c>
       <c r="C111" t="str">
         <v/>
@@ -1958,13 +1958,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B112" t="str">
-        <v>Ellips-TG8</v>
+        <v>TG5TreugDarkGrey</v>
       </c>
       <c r="C112" t="str">
         <v/>
       </c>
       <c r="D112">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="113">
@@ -1972,13 +1972,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B113" t="str">
-        <v>ConfettiViolet-TG8</v>
+        <v>TG5UrbanDarkGrey</v>
       </c>
       <c r="C113" t="str">
         <v/>
       </c>
       <c r="D113">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="114">
@@ -1986,13 +1986,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B114" t="str">
-        <v>ValenciaBlueLiliac-TG8</v>
+        <v>TG5VernisageLightGrey</v>
       </c>
       <c r="C114" t="str">
         <v/>
       </c>
       <c r="D114">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="115">
@@ -2000,7 +2000,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B115" t="str">
-        <v>StripeSilver-TG8</v>
+        <v>TG5ViolettaLavand</v>
       </c>
       <c r="C115" t="str">
         <v/>
@@ -2014,13 +2014,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B116" t="str">
-        <v>TattersolLightGrey-TG8</v>
+        <v>TG5TheoremaBej</v>
       </c>
       <c r="C116" t="str">
         <v/>
       </c>
       <c r="D116">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="117">
@@ -2028,13 +2028,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B117" t="str">
-        <v>FleurTurquoise-TG8</v>
+        <v>TG5LabuBej</v>
       </c>
       <c r="C117" t="str">
         <v/>
       </c>
       <c r="D117">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="118">
@@ -2042,7 +2042,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B118" t="str">
-        <v>EucaliptusPink-TG8</v>
+        <v>TG5FidgieBlack</v>
       </c>
       <c r="C118" t="str">
         <v/>
@@ -2056,7 +2056,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B119" t="str">
-        <v>MramorGrey-TG8</v>
+        <v>TG5ColiseumBZ</v>
       </c>
       <c r="C119" t="str">
         <v/>
@@ -2070,7 +2070,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B120" t="str">
-        <v>CubicGrey-TG8</v>
+        <v>TG5ConfettiViolet</v>
       </c>
       <c r="C120" t="str">
         <v/>
@@ -2084,13 +2084,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B121" t="str">
-        <v>FeeriyaBluePurple-TG8</v>
+        <v>TG5GraciaGray</v>
       </c>
       <c r="C121" t="str">
         <v/>
       </c>
       <c r="D121">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="122">
@@ -2098,7 +2098,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B122" t="str">
-        <v>WesternOrange-TG8</v>
+        <v>TG5MagicBordo</v>
       </c>
       <c r="C122" t="str">
         <v/>
@@ -2112,7 +2112,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B123" t="str">
-        <v>TropicanaBej-TG8</v>
+        <v>TG5TaboLapkaPink</v>
       </c>
       <c r="C123" t="str">
         <v/>
@@ -2126,13 +2126,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B124" t="str">
-        <v>TropicanaGreyTurquoise-TG8</v>
+        <v>TG5ValsBZLightBlue</v>
       </c>
       <c r="C124" t="str">
         <v/>
       </c>
       <c r="D124">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="125">
@@ -2140,7 +2140,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B125" t="str">
-        <v>MonblanColour-TG8</v>
+        <v>TG5MishkiTeddiBrown</v>
       </c>
       <c r="C125" t="str">
         <v/>
@@ -2154,7 +2154,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B126" t="str">
-        <v>Raduga-TG8</v>
+        <v>TG5VenzelBlueBej</v>
       </c>
       <c r="C126" t="str">
         <v/>
@@ -2168,13 +2168,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B127" t="str">
-        <v>KaramelBZ-TG8</v>
+        <v>TG5MishkiWhitePink</v>
       </c>
       <c r="C127" t="str">
         <v/>
       </c>
       <c r="D127">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="128">
@@ -2182,7 +2182,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B128" t="str">
-        <v>TattersolGreyBeige-TG8</v>
+        <v>TG5ZaikiWhitePink</v>
       </c>
       <c r="C128" t="str">
         <v/>
@@ -2196,7 +2196,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B129" t="str">
-        <v>PoligonsDeepBlue-TG8</v>
+        <v>TG5PolosatieMishkiGreen</v>
       </c>
       <c r="C129" t="str">
         <v/>
@@ -2210,13 +2210,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B130" t="str">
-        <v>TotemYellow-TG8</v>
+        <v>TG5ZaichishkiBeige</v>
       </c>
       <c r="C130" t="str">
         <v/>
       </c>
       <c r="D130">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="131">
@@ -2224,7 +2224,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B131" t="str">
-        <v>ContourBZ-TG8</v>
+        <v>TG5TattersolLightGray</v>
       </c>
       <c r="C131" t="str">
         <v/>
@@ -2238,7 +2238,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B132" t="str">
-        <v>CubicBej-TG8</v>
+        <v>TG5PerfectAntracit</v>
       </c>
       <c r="C132" t="str">
         <v/>
@@ -2252,7 +2252,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B133" t="str">
-        <v>RomanticLightBlue-TG8</v>
+        <v>TG5GalaxyBlue</v>
       </c>
       <c r="C133" t="str">
         <v/>
@@ -2266,7 +2266,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B134" t="str">
-        <v>ConfettiBrown-TG8</v>
+        <v>TG5HollywoodBrown</v>
       </c>
       <c r="C134" t="str">
         <v/>
@@ -2280,7 +2280,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B135" t="str">
-        <v>TropicanaBlack-TG8</v>
+        <v>TG5WesternSeaWave</v>
       </c>
       <c r="C135" t="str">
         <v/>
@@ -2294,13 +2294,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B136" t="str">
-        <v>Madlen-TG8</v>
+        <v>TG5EucaliptBZGreen</v>
       </c>
       <c r="C136" t="str">
         <v/>
       </c>
       <c r="D136">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="137">
@@ -2308,7 +2308,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B137" t="str">
-        <v>RomanticBlue-TG8</v>
+        <v>TG5NeonCatsColor</v>
       </c>
       <c r="C137" t="str">
         <v/>
@@ -2322,7 +2322,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B138" t="str">
-        <v>MramorTurquoise-TG8</v>
+        <v>TG5GraciaBZGreen</v>
       </c>
       <c r="C138" t="str">
         <v/>
@@ -2336,13 +2336,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B139" t="str">
-        <v>SymphonyFist-TG8</v>
+        <v>TG5UrbanBZGray</v>
       </c>
       <c r="C139" t="str">
         <v/>
       </c>
       <c r="D139">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="140">
@@ -2350,7 +2350,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B140" t="str">
-        <v>SmilesBZ-TG8</v>
+        <v>TG5GraphicaTurq</v>
       </c>
       <c r="C140" t="str">
         <v/>
@@ -2364,7 +2364,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B141" t="str">
-        <v>TG3ViolettaLavand</v>
+        <v>TG5CvetenieGreyBlue</v>
       </c>
       <c r="C141" t="str">
         <v/>
@@ -2378,7 +2378,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B142" t="str">
-        <v>TG3AmazonkaBZ</v>
+        <v>TG5ListopadBZgrey</v>
       </c>
       <c r="C142" t="str">
         <v/>
@@ -2392,7 +2392,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B143" t="str">
-        <v>TG3AmourBeloZemel</v>
+        <v>TG5SymphonyFist</v>
       </c>
       <c r="C143" t="str">
         <v/>
@@ -2406,13 +2406,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B144" t="str">
-        <v>TG3MagicBordo</v>
+        <v>TG5MramorGrey</v>
       </c>
       <c r="C144" t="str">
         <v/>
       </c>
       <c r="D144">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="145">
@@ -2420,13 +2420,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B145" t="str">
-        <v>TG3RadugaBej</v>
+        <v>TG5TatterlineBej</v>
       </c>
       <c r="C145" t="str">
         <v/>
       </c>
       <c r="D145">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="146">
@@ -2434,7 +2434,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B146" t="str">
-        <v>TG3TucansGreen</v>
+        <v>TG5StambulLightBlue</v>
       </c>
       <c r="C146" t="str">
         <v/>
@@ -2448,13 +2448,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B147" t="str">
-        <v>ViolettaLavand-TG8</v>
+        <v>TG5FidgieBZ</v>
       </c>
       <c r="C147" t="str">
         <v/>
       </c>
       <c r="D147">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="148">
@@ -2462,13 +2462,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B148" t="str">
-        <v>AmazonkaBZ-TG8</v>
+        <v>TG5PoligonsFist</v>
       </c>
       <c r="C148" t="str">
         <v/>
       </c>
       <c r="D148">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="149">
@@ -2476,13 +2476,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B149" t="str">
-        <v>AmourBZ-TG8</v>
+        <v>TG5MishkiTeddiBej</v>
       </c>
       <c r="C149" t="str">
         <v/>
       </c>
       <c r="D149">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="150">
@@ -2490,7 +2490,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B150" t="str">
-        <v>MagicBordo-TG8</v>
+        <v>TG5VernisageLightBlue</v>
       </c>
       <c r="C150" t="str">
         <v/>
@@ -2504,13 +2504,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B151" t="str">
-        <v>RadugaBej-TG8</v>
+        <v>TG5PoligonsDeepBlue</v>
       </c>
       <c r="C151" t="str">
         <v/>
       </c>
       <c r="D151">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="152">
@@ -2518,13 +2518,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B152" t="str">
-        <v>TucansGreen-TG8</v>
+        <v>TG5YablonevCvetPink</v>
       </c>
       <c r="C152" t="str">
         <v/>
       </c>
       <c r="D152">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="153">
@@ -2532,648 +2532,18 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B153" t="str">
-        <v>TG3PositiveLightGrey</v>
+        <v>TG5StambulGreen</v>
       </c>
       <c r="C153" t="str">
         <v/>
       </c>
       <c r="D153">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B154" t="str">
-        <v>TG3GlorisGrey</v>
-      </c>
-      <c r="C154" t="str">
-        <v/>
-      </c>
-      <c r="D154">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B155" t="str">
-        <v>TG3LetniySadBZ</v>
-      </c>
-      <c r="C155" t="str">
-        <v/>
-      </c>
-      <c r="D155">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B156" t="str">
-        <v>TG3BestFriendBej</v>
-      </c>
-      <c r="C156" t="str">
-        <v/>
-      </c>
-      <c r="D156">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B157" t="str">
-        <v>TG3Jaklin</v>
-      </c>
-      <c r="C157" t="str">
-        <v/>
-      </c>
-      <c r="D157">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B158" t="str">
-        <v>TG3LazurBZLightBlue</v>
-      </c>
-      <c r="C158" t="str">
-        <v/>
-      </c>
-      <c r="D158">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B159" t="str">
-        <v>TG2VizantBejPink33</v>
-      </c>
-      <c r="C159" t="str">
-        <v/>
-      </c>
-      <c r="D159">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B160" t="str">
-        <v>TG2GalaxyChoko33</v>
-      </c>
-      <c r="C160" t="str">
-        <v/>
-      </c>
-      <c r="D160">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B161" t="str">
-        <v>TG2JungleTurqGreen33</v>
-      </c>
-      <c r="C161" t="str">
-        <v/>
-      </c>
-      <c r="D161">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B162" t="str">
-        <v>TG2ListopadBZgrey33</v>
-      </c>
-      <c r="C162" t="str">
-        <v/>
-      </c>
-      <c r="D162">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B163" t="str">
-        <v>TG2MilflerBZlightBlue33</v>
-      </c>
-      <c r="C163" t="str">
-        <v/>
-      </c>
-      <c r="D163">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B164" t="str">
-        <v>TG2MilflerBZpink33</v>
-      </c>
-      <c r="C164" t="str">
-        <v/>
-      </c>
-      <c r="D164">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B165" t="str">
-        <v>TG2TartanBZpink33</v>
-      </c>
-      <c r="C165" t="str">
-        <v/>
-      </c>
-      <c r="D165">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B166" t="str">
-        <v>TG2TeoremaGrey33</v>
-      </c>
-      <c r="C166" t="str">
-        <v/>
-      </c>
-      <c r="D166">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B167" t="str">
-        <v>VizantBejPink-TG8</v>
-      </c>
-      <c r="C167" t="str">
-        <v/>
-      </c>
-      <c r="D167">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B168" t="str">
-        <v>GalaxyChoko-TG8</v>
-      </c>
-      <c r="C168" t="str">
-        <v/>
-      </c>
-      <c r="D168">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B169" t="str">
-        <v>JungleTurqGreen-TG8</v>
-      </c>
-      <c r="C169" t="str">
-        <v/>
-      </c>
-      <c r="D169">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B170" t="str">
-        <v>ListopadBZgrey-TG8</v>
-      </c>
-      <c r="C170" t="str">
-        <v/>
-      </c>
-      <c r="D170">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B171" t="str">
-        <v>MilflerBZlightBlue-TG8</v>
-      </c>
-      <c r="C171" t="str">
-        <v/>
-      </c>
-      <c r="D171">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B172" t="str">
-        <v>MilflerBZpink-TG8</v>
-      </c>
-      <c r="C172" t="str">
-        <v/>
-      </c>
-      <c r="D172">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B173" t="str">
-        <v>TartanBZpink-TG8</v>
-      </c>
-      <c r="C173" t="str">
-        <v/>
-      </c>
-      <c r="D173">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B174" t="str">
-        <v>TeoremaGrey-TG8</v>
-      </c>
-      <c r="C174" t="str">
-        <v/>
-      </c>
-      <c r="D174">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B175" t="str">
-        <v>TG2CubicBordo</v>
-      </c>
-      <c r="C175" t="str">
-        <v/>
-      </c>
-      <c r="D175">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B176" t="str">
-        <v>CubicBordo-TG8</v>
-      </c>
-      <c r="C176" t="str">
-        <v/>
-      </c>
-      <c r="D176">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B177" t="str">
-        <v>TG1AvangardBZgrey</v>
-      </c>
-      <c r="C177" t="str">
-        <v/>
-      </c>
-      <c r="D177">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B178" t="str">
-        <v>TG1TatterlineBej</v>
-      </c>
-      <c r="C178" t="str">
-        <v/>
-      </c>
-      <c r="D178">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B179" t="str">
-        <v>TG1TheoremaBej</v>
-      </c>
-      <c r="C179" t="str">
-        <v/>
-      </c>
-      <c r="D179">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B180" t="str">
-        <v>TG1UrbanDarkGrey</v>
-      </c>
-      <c r="C180" t="str">
-        <v/>
-      </c>
-      <c r="D180">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B181" t="str">
-        <v>TatterlineBej-TG8</v>
-      </c>
-      <c r="C181" t="str">
-        <v/>
-      </c>
-      <c r="D181">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B182" t="str">
-        <v>UrbanDarkGrey-TG8</v>
-      </c>
-      <c r="C182" t="str">
-        <v/>
-      </c>
-      <c r="D182">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B183" t="str">
-        <v>AvangardBZgrey-TG8</v>
-      </c>
-      <c r="C183" t="str">
-        <v/>
-      </c>
-      <c r="D183">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B184" t="str">
-        <v>TheoremaBej-TG8</v>
-      </c>
-      <c r="C184" t="str">
-        <v/>
-      </c>
-      <c r="D184">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B185" t="str">
-        <v>LavandBuketBZ-TG8</v>
-      </c>
-      <c r="C185" t="str">
-        <v/>
-      </c>
-      <c r="D185">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B186" t="str">
-        <v>LineBlue-TG8</v>
-      </c>
-      <c r="C186" t="str">
-        <v/>
-      </c>
-      <c r="D186">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B187" t="str">
-        <v>UrbanBZgray-TG8</v>
-      </c>
-      <c r="C187" t="str">
-        <v/>
-      </c>
-      <c r="D187">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B188" t="str">
-        <v>TG1LineBlue</v>
-      </c>
-      <c r="C188" t="str">
-        <v/>
-      </c>
-      <c r="D188">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B189" t="str">
-        <v>TG1UrbanBZGray</v>
-      </c>
-      <c r="C189" t="str">
-        <v/>
-      </c>
-      <c r="D189">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B190" t="str">
-        <v>TG1LavandBuketBZ</v>
-      </c>
-      <c r="C190" t="str">
-        <v/>
-      </c>
-      <c r="D190">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B191" t="str">
-        <v>TG2ConfettiViolet</v>
-      </c>
-      <c r="C191" t="str">
-        <v/>
-      </c>
-      <c r="D191">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B192" t="str">
-        <v>TG2ConfettiBlueLilac</v>
-      </c>
-      <c r="C192" t="str">
-        <v/>
-      </c>
-      <c r="D192">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B193" t="str">
-        <v>TG2ConfettiTurquoise</v>
-      </c>
-      <c r="C193" t="str">
-        <v/>
-      </c>
-      <c r="D193">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B194" t="str">
-        <v>TG2VernisageLightGray</v>
-      </c>
-      <c r="C194" t="str">
-        <v/>
-      </c>
-      <c r="D194">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B195" t="str">
-        <v>TG2MargaritkaViolet</v>
-      </c>
-      <c r="C195" t="str">
-        <v/>
-      </c>
-      <c r="D195">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B196" t="str">
-        <v>TG2KavalkadaBZGray</v>
-      </c>
-      <c r="C196" t="str">
-        <v/>
-      </c>
-      <c r="D196">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="197">
-      <c r="A197" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B197" t="str">
-        <v>TG2ValentinkaBeige</v>
-      </c>
-      <c r="C197" t="str">
-        <v/>
-      </c>
-      <c r="D197">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="198">
-      <c r="A198" t="str">
-        <v>СЦ (Коляново) (1020002072018000)</v>
-      </c>
-      <c r="B198" t="str">
-        <v>TG2IndustrialGrayYellow</v>
-      </c>
-      <c r="C198" t="str">
-        <v/>
-      </c>
-      <c r="D198">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D198"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D153"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix stringToInt func, inscreased output stocks, decreased supplier's stocks limit
</commit_message>
<xml_diff>
--- a/data/ready_stocks/galtex-ozon-stocks-updated.xlsx
+++ b/data/ready_stocks/galtex-ozon-stocks-updated.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D153"/>
+  <dimension ref="A1:D166"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -418,13 +418,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B2" t="str">
-        <v>TG5CircusWhiteEarth150/50</v>
+        <v>TG5WesternGrey150/50</v>
       </c>
       <c r="C2" t="str">
         <v/>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3">
@@ -432,7 +432,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B3" t="str">
-        <v>TG5losang150/50</v>
+        <v>TG5CircusWhiteEarth150/50</v>
       </c>
       <c r="C3" t="str">
         <v/>
@@ -446,7 +446,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B4" t="str">
-        <v>TG5GraphicOrange150/50</v>
+        <v>TG5losang150/50</v>
       </c>
       <c r="C4" t="str">
         <v/>
@@ -460,7 +460,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B5" t="str">
-        <v>TG5EucaliptPink150/50</v>
+        <v>TG5GraphicOrange150/50</v>
       </c>
       <c r="C5" t="str">
         <v/>
@@ -474,7 +474,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B6" t="str">
-        <v>TG5stripeViol150/50</v>
+        <v>TG5EucaliptPink150/50</v>
       </c>
       <c r="C6" t="str">
         <v/>
@@ -488,7 +488,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B7" t="str">
-        <v>TG5CatHomeDeepBlue150/50</v>
+        <v>TG5stripeViol150/50</v>
       </c>
       <c r="C7" t="str">
         <v/>
@@ -502,7 +502,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B8" t="str">
-        <v>TG5FlowerSakurLavand150/50</v>
+        <v>TG5CatHomeDeepBlue150/50</v>
       </c>
       <c r="C8" t="str">
         <v/>
@@ -516,13 +516,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B9" t="str">
-        <v>TG5kotbaton150/50</v>
+        <v>TG5FlowerSakurLavand150/50</v>
       </c>
       <c r="C9" t="str">
         <v/>
       </c>
       <c r="D9">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -530,13 +530,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B10" t="str">
-        <v>TG5BibigonBej150/50</v>
+        <v>TG5kotbaton150/50</v>
       </c>
       <c r="C10" t="str">
         <v/>
       </c>
       <c r="D10">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11">
@@ -544,7 +544,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B11" t="str">
-        <v>TG5GraphicChoco150/50</v>
+        <v>TG5BibigonBej150/50</v>
       </c>
       <c r="C11" t="str">
         <v/>
@@ -558,7 +558,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B12" t="str">
-        <v>TG5CatHomeDeepGrey150/50</v>
+        <v>TG5GraphicChoco150/50</v>
       </c>
       <c r="C12" t="str">
         <v/>
@@ -572,13 +572,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B13" t="str">
-        <v>TG5gta150/50</v>
+        <v>TG5CatHomeDeepGrey150/50</v>
       </c>
       <c r="C13" t="str">
         <v/>
       </c>
       <c r="D13">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -586,13 +586,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B14" t="str">
-        <v>TG5stripeChoco150/50</v>
+        <v>TG5gta150/50</v>
       </c>
       <c r="C14" t="str">
         <v/>
       </c>
       <c r="D14">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15">
@@ -600,7 +600,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B15" t="str">
-        <v>TG5EucaliptBlue150/50</v>
+        <v>TG5stripeChoco150/50</v>
       </c>
       <c r="C15" t="str">
         <v/>
@@ -614,7 +614,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B16" t="str">
-        <v>TG5Grani</v>
+        <v>TG5EucaliptBlue150/50</v>
       </c>
       <c r="C16" t="str">
         <v/>
@@ -628,7 +628,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B17" t="str">
-        <v>TG5TreugolnikiTurquoise</v>
+        <v>TG5Grani</v>
       </c>
       <c r="C17" t="str">
         <v/>
@@ -642,7 +642,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B18" t="str">
-        <v>TG5TattersolBZ</v>
+        <v>TG5TreugolnikiTurquoise</v>
       </c>
       <c r="C18" t="str">
         <v/>
@@ -656,7 +656,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B19" t="str">
-        <v>TG5SymphonyPowder</v>
+        <v>TG5TattersolBZ</v>
       </c>
       <c r="C19" t="str">
         <v/>
@@ -670,7 +670,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B20" t="str">
-        <v>TG5HollywoodDarkBeige</v>
+        <v>TG5SymphonyPowder</v>
       </c>
       <c r="C20" t="str">
         <v/>
@@ -684,7 +684,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B21" t="str">
-        <v>TG5animeDarkGrey</v>
+        <v>TG5HollywoodDarkBeige</v>
       </c>
       <c r="C21" t="str">
         <v/>
@@ -698,7 +698,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B22" t="str">
-        <v>TG5FlyBZ</v>
+        <v>TG5animeDarkGrey</v>
       </c>
       <c r="C22" t="str">
         <v/>
@@ -712,13 +712,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B23" t="str">
-        <v>TG5BeskonechnostBZ</v>
+        <v>TG5FlyBZ</v>
       </c>
       <c r="C23" t="str">
         <v/>
       </c>
       <c r="D23">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -726,13 +726,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B24" t="str">
-        <v>TG5ZavitokLavanda</v>
+        <v>TG5BeskonechnostBZ</v>
       </c>
       <c r="C24" t="str">
         <v/>
       </c>
       <c r="D24">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="25">
@@ -740,7 +740,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B25" t="str">
-        <v>TG5KletochkaTurquoise</v>
+        <v>TG5ZavitokLavanda</v>
       </c>
       <c r="C25" t="str">
         <v/>
@@ -754,7 +754,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B26" t="str">
-        <v>TG5StrekoziGreyBeige</v>
+        <v>TG5KletochkaTurquoise</v>
       </c>
       <c r="C26" t="str">
         <v/>
@@ -768,7 +768,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B27" t="str">
-        <v>TG5VichyLightBlue</v>
+        <v>TG5StrekoziGreyBeige</v>
       </c>
       <c r="C27" t="str">
         <v/>
@@ -782,7 +782,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B28" t="str">
-        <v>TG5GlorisGrey</v>
+        <v>TG5VichyLightBlue</v>
       </c>
       <c r="C28" t="str">
         <v/>
@@ -796,13 +796,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B29" t="str">
-        <v>TG5LabirintBrown</v>
+        <v>TG5GlorisGrey</v>
       </c>
       <c r="C29" t="str">
         <v/>
       </c>
       <c r="D29">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -810,13 +810,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B30" t="str">
-        <v>TG5SymphonyLightBlue</v>
+        <v>TG5LabirintBrown</v>
       </c>
       <c r="C30" t="str">
         <v/>
       </c>
       <c r="D30">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="31">
@@ -824,7 +824,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B31" t="str">
-        <v>TG5ContourBeige</v>
+        <v>TG5SymphonyLightBlue</v>
       </c>
       <c r="C31" t="str">
         <v/>
@@ -838,13 +838,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B32" t="str">
-        <v>TG5TropicTurquoise</v>
+        <v>TG5ContourBeige</v>
       </c>
       <c r="C32" t="str">
         <v/>
       </c>
       <c r="D32">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -852,13 +852,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B33" t="str">
-        <v>TG5SladkieSniGrafit</v>
+        <v>TG5TropicTurquoise</v>
       </c>
       <c r="C33" t="str">
         <v/>
       </c>
       <c r="D33">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="34">
@@ -866,7 +866,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B34" t="str">
-        <v>TG5ShtrikhiMocco</v>
+        <v>TG5SladkieSniGrafit</v>
       </c>
       <c r="C34" t="str">
         <v/>
@@ -880,7 +880,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B35" t="str">
-        <v>TG5BibigonGreen</v>
+        <v>TG5ShtrikhiMocco</v>
       </c>
       <c r="C35" t="str">
         <v/>
@@ -894,7 +894,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B36" t="str">
-        <v>TG5TropicanaGreyTurquoise</v>
+        <v>TG5BibigonGreen</v>
       </c>
       <c r="C36" t="str">
         <v/>
@@ -908,7 +908,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B37" t="str">
-        <v>TG5ZavitokLightBlue</v>
+        <v>TG5TropicanaGreyTurquoise</v>
       </c>
       <c r="C37" t="str">
         <v/>
@@ -922,13 +922,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B38" t="str">
-        <v>TG5PandaBeige</v>
+        <v>TG5ZavitokLightBlue</v>
       </c>
       <c r="C38" t="str">
         <v/>
       </c>
       <c r="D38">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="39">
@@ -936,13 +936,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B39" t="str">
-        <v>TG5QuestBZGreen</v>
+        <v>TG5PandaBeige</v>
       </c>
       <c r="C39" t="str">
         <v/>
       </c>
       <c r="D39">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -950,13 +950,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B40" t="str">
-        <v>TG5BogemaTurquoise</v>
+        <v>TG5QuestBZGreen</v>
       </c>
       <c r="C40" t="str">
         <v/>
       </c>
       <c r="D40">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="41">
@@ -964,13 +964,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B41" t="str">
-        <v>TG5StepBlack</v>
+        <v>TG5BogemaTurquoise</v>
       </c>
       <c r="C41" t="str">
         <v/>
       </c>
       <c r="D41">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="42">
@@ -978,7 +978,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B42" t="str">
-        <v>TG5RozaPink</v>
+        <v>TG5StepBlack</v>
       </c>
       <c r="C42" t="str">
         <v/>
@@ -992,7 +992,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B43" t="str">
-        <v>TG5StripePowder</v>
+        <v>TG5RozaPink</v>
       </c>
       <c r="C43" t="str">
         <v/>
@@ -1006,13 +1006,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B44" t="str">
-        <v>TG5StrekoziMint</v>
+        <v>TG5StripePowder</v>
       </c>
       <c r="C44" t="str">
         <v/>
       </c>
       <c r="D44">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -1020,13 +1020,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B45" t="str">
-        <v>TG5TropicanaBej</v>
+        <v>TG5StrekoziMint</v>
       </c>
       <c r="C45" t="str">
         <v/>
       </c>
       <c r="D45">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="46">
@@ -1034,7 +1034,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B46" t="str">
-        <v>TG5GoodNightLightBlue</v>
+        <v>TG5TropicanaBej</v>
       </c>
       <c r="C46" t="str">
         <v/>
@@ -1048,7 +1048,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B47" t="str">
-        <v>TG5MishkiWhiteGreen</v>
+        <v>TG5GoodNightLightBlue</v>
       </c>
       <c r="C47" t="str">
         <v/>
@@ -1062,7 +1062,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B48" t="str">
-        <v>TG5DialoguePink</v>
+        <v>TG5MishkiWhiteGreen</v>
       </c>
       <c r="C48" t="str">
         <v/>
@@ -1076,13 +1076,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B49" t="str">
-        <v>TG5PolosatieMishkiBZ</v>
+        <v>TG5DialoguePink</v>
       </c>
       <c r="C49" t="str">
         <v/>
       </c>
       <c r="D49">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -1090,13 +1090,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B50" t="str">
-        <v>TG5StarNightBlack</v>
+        <v>TG5PolosatieMishkiBZ</v>
       </c>
       <c r="C50" t="str">
         <v/>
       </c>
       <c r="D50">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="51">
@@ -1104,13 +1104,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B51" t="str">
-        <v>TG5Kotovasia</v>
+        <v>TG5StarNightBlack</v>
       </c>
       <c r="C51" t="str">
         <v/>
       </c>
       <c r="D51">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="52">
@@ -1118,13 +1118,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B52" t="str">
-        <v>TG5StripeSilver</v>
+        <v>TG5Kotovasia</v>
       </c>
       <c r="C52" t="str">
         <v/>
       </c>
       <c r="D52">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="53">
@@ -1132,13 +1132,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B53" t="str">
-        <v>TG5ZaikiWhiteBlue</v>
+        <v>TG5StripeSilver</v>
       </c>
       <c r="C53" t="str">
         <v/>
       </c>
       <c r="D53">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54">
@@ -1146,13 +1146,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B54" t="str">
-        <v>TG5KletochkaMint</v>
+        <v>TG5ZaikiWhiteBlue</v>
       </c>
       <c r="C54" t="str">
         <v/>
       </c>
       <c r="D54">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="55">
@@ -1160,13 +1160,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B55" t="str">
-        <v>TG5MramorTurquoise</v>
+        <v>TG5KletochkaMint</v>
       </c>
       <c r="C55" t="str">
         <v/>
       </c>
       <c r="D55">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="56">
@@ -1174,13 +1174,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B56" t="str">
-        <v>TG5ArabeskiLightBlue</v>
+        <v>TG5MramorTurquoise</v>
       </c>
       <c r="C56" t="str">
         <v/>
       </c>
       <c r="D56">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="57">
@@ -1188,7 +1188,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B57" t="str">
-        <v>TG5MishkiWhiteYellow</v>
+        <v>TG5ArabeskiLightBlue</v>
       </c>
       <c r="C57" t="str">
         <v/>
@@ -1202,7 +1202,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B58" t="str">
-        <v>TG5GooseOtosplus</v>
+        <v>TG5MishkiWhiteYellow</v>
       </c>
       <c r="C58" t="str">
         <v/>
@@ -1216,13 +1216,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B59" t="str">
-        <v>TG5DialogueTurquoise</v>
+        <v>TG5GooseOtosplus</v>
       </c>
       <c r="C59" t="str">
         <v/>
       </c>
       <c r="D59">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="60">
@@ -1230,7 +1230,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B60" t="str">
-        <v>TG5Florans</v>
+        <v>TG5DialogueTurquoise</v>
       </c>
       <c r="C60" t="str">
         <v/>
@@ -1244,7 +1244,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B61" t="str">
-        <v>TG5ZavitokChoco</v>
+        <v>TG5Florans</v>
       </c>
       <c r="C61" t="str">
         <v/>
@@ -1258,7 +1258,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B62" t="str">
-        <v>TG5BanansGreen</v>
+        <v>TG5ZavitokChoco</v>
       </c>
       <c r="C62" t="str">
         <v/>
@@ -1272,7 +1272,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B63" t="str">
-        <v>TG5SmilesGrey</v>
+        <v>TG5BanansGreen</v>
       </c>
       <c r="C63" t="str">
         <v/>
@@ -1286,7 +1286,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B64" t="str">
-        <v>TG5StrekoziLightBlue</v>
+        <v>TG5SmilesGrey</v>
       </c>
       <c r="C64" t="str">
         <v/>
@@ -1300,7 +1300,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B65" t="str">
-        <v>TG5MishkiWhiteBlue</v>
+        <v>TG5StrekoziLightBlue</v>
       </c>
       <c r="C65" t="str">
         <v/>
@@ -1314,7 +1314,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B66" t="str">
-        <v>TG5ValenciaBlueLiliac</v>
+        <v>TG5MishkiWhiteBlue</v>
       </c>
       <c r="C66" t="str">
         <v/>
@@ -1328,13 +1328,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B67" t="str">
-        <v>TG5LondonTurquoise</v>
+        <v>TG5ValenciaBlueLiliac</v>
       </c>
       <c r="C67" t="str">
         <v/>
       </c>
       <c r="D67">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="68">
@@ -1342,13 +1342,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B68" t="str">
-        <v>TG5TropicanaBlack</v>
+        <v>TG5LondonTurquoise</v>
       </c>
       <c r="C68" t="str">
         <v/>
       </c>
       <c r="D68">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="69">
@@ -1356,13 +1356,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B69" t="str">
-        <v>TG5WesternPowder</v>
+        <v>TG5TropicanaBlack</v>
       </c>
       <c r="C69" t="str">
         <v/>
       </c>
       <c r="D69">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="70">
@@ -1370,13 +1370,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B70" t="str">
-        <v>TG5ValenciaGreenTurq</v>
+        <v>TG5WesternPowder</v>
       </c>
       <c r="C70" t="str">
         <v/>
       </c>
       <c r="D70">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="71">
@@ -1384,7 +1384,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B71" t="str">
-        <v>TG5ZooparkGreen</v>
+        <v>TG5ValenciaGreenTurq</v>
       </c>
       <c r="C71" t="str">
         <v/>
@@ -1398,7 +1398,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B72" t="str">
-        <v>TG5VenzelBej</v>
+        <v>TG5ZooparkGreen</v>
       </c>
       <c r="C72" t="str">
         <v/>
@@ -1412,7 +1412,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B73" t="str">
-        <v>TG5ValenciaBej</v>
+        <v>TG5VenzelBej</v>
       </c>
       <c r="C73" t="str">
         <v/>
@@ -1426,7 +1426,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B74" t="str">
-        <v>TG5ValenciaBZ</v>
+        <v>TG5ValenciaBej</v>
       </c>
       <c r="C74" t="str">
         <v/>
@@ -1440,13 +1440,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B75" t="str">
-        <v>TG5TattersolGreyBej</v>
+        <v>TG5ValenciaBZ</v>
       </c>
       <c r="C75" t="str">
         <v/>
       </c>
       <c r="D75">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76">
@@ -1454,13 +1454,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B76" t="str">
-        <v>TG5StarLightGrey</v>
+        <v>TG5TattersolGreyBej</v>
       </c>
       <c r="C76" t="str">
         <v/>
       </c>
       <c r="D76">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="77">
@@ -1468,7 +1468,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B77" t="str">
-        <v>TG5StarTurquoise</v>
+        <v>TG5StarLightGrey</v>
       </c>
       <c r="C77" t="str">
         <v/>
@@ -1482,7 +1482,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B78" t="str">
-        <v>TG5GTAColor</v>
+        <v>TG5StarTurquoise</v>
       </c>
       <c r="C78" t="str">
         <v/>
@@ -1496,7 +1496,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B79" t="str">
-        <v>TG5PerfectNiagara</v>
+        <v>TG5GTAColor</v>
       </c>
       <c r="C79" t="str">
         <v/>
@@ -1510,13 +1510,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B80" t="str">
-        <v>TG5IllusionGrey</v>
+        <v>TG5PerfectNiagara</v>
       </c>
       <c r="C80" t="str">
         <v/>
       </c>
       <c r="D80">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="81">
@@ -1524,13 +1524,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B81" t="str">
-        <v>TG5LabirintVasilek</v>
+        <v>TG5IllusionGrey</v>
       </c>
       <c r="C81" t="str">
         <v/>
       </c>
       <c r="D81">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="82">
@@ -1538,13 +1538,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B82" t="str">
-        <v>TG5ContourLightGrey</v>
+        <v>TG5LabirintVasilek</v>
       </c>
       <c r="C82" t="str">
         <v/>
       </c>
       <c r="D82">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="83">
@@ -1552,13 +1552,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B83" t="str">
-        <v>TG5Colibri</v>
+        <v>TG5ContourLightGrey</v>
       </c>
       <c r="C83" t="str">
         <v/>
       </c>
       <c r="D83">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="84">
@@ -1566,7 +1566,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B84" t="str">
-        <v>TG5SmilesBZWhite</v>
+        <v>TG5Colibri</v>
       </c>
       <c r="C84" t="str">
         <v/>
@@ -1580,7 +1580,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B85" t="str">
-        <v>TG5PoligonSeaWave</v>
+        <v>TG5SmilesBZWhite</v>
       </c>
       <c r="C85" t="str">
         <v/>
@@ -1594,7 +1594,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B86" t="str">
-        <v>TG5LetniySad</v>
+        <v>TG5PoligonSeaWave</v>
       </c>
       <c r="C86" t="str">
         <v/>
@@ -1608,7 +1608,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B87" t="str">
-        <v>TG5KletochkaBej</v>
+        <v>TG5LetniySad</v>
       </c>
       <c r="C87" t="str">
         <v/>
@@ -1622,7 +1622,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B88" t="str">
-        <v>TG5Creative</v>
+        <v>TG5KletochkaBej</v>
       </c>
       <c r="C88" t="str">
         <v/>
@@ -1636,13 +1636,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B89" t="str">
-        <v>TG5SozvezdieBlack</v>
+        <v>TG5Creative</v>
       </c>
       <c r="C89" t="str">
         <v/>
       </c>
       <c r="D89">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="90">
@@ -1650,13 +1650,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B90" t="str">
-        <v>TG5OwlHomeBejPink</v>
+        <v>TG5SozvezdieBlack</v>
       </c>
       <c r="C90" t="str">
         <v/>
       </c>
       <c r="D90">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="91">
@@ -1664,13 +1664,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B91" t="str">
-        <v>TG5FloransBZsiren</v>
+        <v>TG5OwlHomeBejPink</v>
       </c>
       <c r="C91" t="str">
         <v/>
       </c>
       <c r="D91">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="92">
@@ -1678,7 +1678,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B92" t="str">
-        <v>TG5BestFriendBej</v>
+        <v>TG5FloransBZsiren</v>
       </c>
       <c r="C92" t="str">
         <v/>
@@ -1692,13 +1692,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B93" t="str">
-        <v>TG5Lyric</v>
+        <v>TG5BestFriendBej</v>
       </c>
       <c r="C93" t="str">
         <v/>
       </c>
       <c r="D93">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="94">
@@ -1706,13 +1706,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B94" t="str">
-        <v>TG5FlowersSakuraPowder</v>
+        <v>TG5Lyric</v>
       </c>
       <c r="C94" t="str">
         <v/>
       </c>
       <c r="D94">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="95">
@@ -1720,13 +1720,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B95" t="str">
-        <v>TG5CapyBej</v>
+        <v>TG5FlowersSakuraPowder</v>
       </c>
       <c r="C95" t="str">
         <v/>
       </c>
       <c r="D95">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="96">
@@ -1734,13 +1734,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B96" t="str">
-        <v>TG5GraciaIzumrud</v>
+        <v>TG5CapyBej</v>
       </c>
       <c r="C96" t="str">
         <v/>
       </c>
       <c r="D96">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="97">
@@ -1748,13 +1748,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B97" t="str">
-        <v>TG5GalaxyChok50</v>
+        <v>TG5GraciaIzumrud</v>
       </c>
       <c r="C97" t="str">
         <v/>
       </c>
       <c r="D97">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="98">
@@ -1762,7 +1762,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B98" t="str">
-        <v>TG5AmourBZ</v>
+        <v>TG5GalaxyChok50</v>
       </c>
       <c r="C98" t="str">
         <v/>
@@ -1776,13 +1776,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B99" t="str">
-        <v>TG5BogemaGrey</v>
+        <v>TG5AmourBZ</v>
       </c>
       <c r="C99" t="str">
         <v/>
       </c>
       <c r="D99">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="100">
@@ -1790,13 +1790,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B100" t="str">
-        <v>TG5ContourDarkGrey</v>
+        <v>TG5BogemaGrey</v>
       </c>
       <c r="C100" t="str">
         <v/>
       </c>
       <c r="D100">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="101">
@@ -1804,13 +1804,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B101" t="str">
-        <v>TG5Fidgie</v>
+        <v>TG5ContourDarkGrey</v>
       </c>
       <c r="C101" t="str">
         <v/>
       </c>
       <c r="D101">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="102">
@@ -1818,7 +1818,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B102" t="str">
-        <v>TG5GraciaBZgrey</v>
+        <v>TG5Fidgie</v>
       </c>
       <c r="C102" t="str">
         <v/>
@@ -1832,7 +1832,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B103" t="str">
-        <v>TG5HollywoodBlue</v>
+        <v>TG5GraciaBZgrey</v>
       </c>
       <c r="C103" t="str">
         <v/>
@@ -1846,13 +1846,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B104" t="str">
-        <v>TG5KotAkula</v>
+        <v>TG5HollywoodBlue</v>
       </c>
       <c r="C104" t="str">
         <v/>
       </c>
       <c r="D104">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="105">
@@ -1860,13 +1860,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B105" t="str">
-        <v>TG5LavandBuketBZ</v>
+        <v>TG5KotAkula</v>
       </c>
       <c r="C105" t="str">
         <v/>
       </c>
       <c r="D105">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="106">
@@ -1874,7 +1874,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B106" t="str">
-        <v>TG5MilflerBZpink</v>
+        <v>TG5LavandBuketBZ</v>
       </c>
       <c r="C106" t="str">
         <v/>
@@ -1888,13 +1888,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B107" t="str">
-        <v>TG5SymphGreyBej</v>
+        <v>TG5MilflerBZpink</v>
       </c>
       <c r="C107" t="str">
         <v/>
       </c>
       <c r="D107">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="108">
@@ -1902,7 +1902,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B108" t="str">
-        <v>TG5TartanBZgrey</v>
+        <v>TG5SymphGreyBej</v>
       </c>
       <c r="C108" t="str">
         <v/>
@@ -1916,7 +1916,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B109" t="str">
-        <v>TG5TheoremBej</v>
+        <v>TG5TartanBZgrey</v>
       </c>
       <c r="C109" t="str">
         <v/>
@@ -1930,7 +1930,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B110" t="str">
-        <v>TG5TheoremGrey</v>
+        <v>TG5TheoremBej</v>
       </c>
       <c r="C110" t="str">
         <v/>
@@ -1944,7 +1944,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B111" t="str">
-        <v>TG5Totem</v>
+        <v>TG5TheoremGrey</v>
       </c>
       <c r="C111" t="str">
         <v/>
@@ -1958,7 +1958,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B112" t="str">
-        <v>TG5TreugDarkGrey</v>
+        <v>TG5Totem</v>
       </c>
       <c r="C112" t="str">
         <v/>
@@ -1972,13 +1972,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B113" t="str">
-        <v>TG5UrbanDarkGrey</v>
+        <v>TG5TreugDarkGrey</v>
       </c>
       <c r="C113" t="str">
         <v/>
       </c>
       <c r="D113">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="114">
@@ -1986,13 +1986,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B114" t="str">
-        <v>TG5VernisageLightGrey</v>
+        <v>TG5UrbanDarkGrey</v>
       </c>
       <c r="C114" t="str">
         <v/>
       </c>
       <c r="D114">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="115">
@@ -2000,13 +2000,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B115" t="str">
-        <v>TG5ViolettaLavand</v>
+        <v>TG5VernisageLightGrey</v>
       </c>
       <c r="C115" t="str">
         <v/>
       </c>
       <c r="D115">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="116">
@@ -2014,13 +2014,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B116" t="str">
-        <v>TG5TheoremaBej</v>
+        <v>TG5ViolettaLavand</v>
       </c>
       <c r="C116" t="str">
         <v/>
       </c>
       <c r="D116">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="117">
@@ -2028,13 +2028,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B117" t="str">
-        <v>TG5LabuBej</v>
+        <v>TG5TheoremaBej</v>
       </c>
       <c r="C117" t="str">
         <v/>
       </c>
       <c r="D117">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="118">
@@ -2042,13 +2042,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B118" t="str">
-        <v>TG5FidgieBlack</v>
+        <v>TG5LabuBej</v>
       </c>
       <c r="C118" t="str">
         <v/>
       </c>
       <c r="D118">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="119">
@@ -2056,13 +2056,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B119" t="str">
-        <v>TG5ColiseumBZ</v>
+        <v>TG5FidgieBlack</v>
       </c>
       <c r="C119" t="str">
         <v/>
       </c>
       <c r="D119">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="120">
@@ -2070,13 +2070,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B120" t="str">
-        <v>TG5ConfettiViolet</v>
+        <v>TG5ColiseumBZ</v>
       </c>
       <c r="C120" t="str">
         <v/>
       </c>
       <c r="D120">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="121">
@@ -2084,13 +2084,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B121" t="str">
-        <v>TG5GraciaGray</v>
+        <v>TG5ConfettiViolet</v>
       </c>
       <c r="C121" t="str">
         <v/>
       </c>
       <c r="D121">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="122">
@@ -2098,13 +2098,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B122" t="str">
-        <v>TG5MagicBordo</v>
+        <v>TG5GraciaGray</v>
       </c>
       <c r="C122" t="str">
         <v/>
       </c>
       <c r="D122">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="123">
@@ -2112,13 +2112,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B123" t="str">
-        <v>TG5TaboLapkaPink</v>
+        <v>TG5MagicBordo</v>
       </c>
       <c r="C123" t="str">
         <v/>
       </c>
       <c r="D123">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="124">
@@ -2126,13 +2126,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B124" t="str">
-        <v>TG5ValsBZLightBlue</v>
+        <v>TG5TaboLapkaPink</v>
       </c>
       <c r="C124" t="str">
         <v/>
       </c>
       <c r="D124">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="125">
@@ -2140,13 +2140,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B125" t="str">
-        <v>TG5MishkiTeddiBrown</v>
+        <v>TG5ValsBZLightBlue</v>
       </c>
       <c r="C125" t="str">
         <v/>
       </c>
       <c r="D125">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="126">
@@ -2154,7 +2154,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B126" t="str">
-        <v>TG5VenzelBlueBej</v>
+        <v>TG5MishkiTeddiBrown</v>
       </c>
       <c r="C126" t="str">
         <v/>
@@ -2168,7 +2168,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B127" t="str">
-        <v>TG5MishkiWhitePink</v>
+        <v>TG5VenzelBlueBej</v>
       </c>
       <c r="C127" t="str">
         <v/>
@@ -2182,13 +2182,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B128" t="str">
-        <v>TG5ZaikiWhitePink</v>
+        <v>TG5MishkiWhitePink</v>
       </c>
       <c r="C128" t="str">
         <v/>
       </c>
       <c r="D128">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="129">
@@ -2196,13 +2196,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B129" t="str">
-        <v>TG5PolosatieMishkiGreen</v>
+        <v>TG5ZaikiWhitePink</v>
       </c>
       <c r="C129" t="str">
         <v/>
       </c>
       <c r="D129">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="130">
@@ -2210,7 +2210,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B130" t="str">
-        <v>TG5ZaichishkiBeige</v>
+        <v>TG5PolosatieMishkiGreen</v>
       </c>
       <c r="C130" t="str">
         <v/>
@@ -2224,7 +2224,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B131" t="str">
-        <v>TG5TattersolLightGray</v>
+        <v>TG5ZaichishkiBeige</v>
       </c>
       <c r="C131" t="str">
         <v/>
@@ -2238,13 +2238,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B132" t="str">
-        <v>TG5PerfectAntracit</v>
+        <v>TG5TattersolLightGray</v>
       </c>
       <c r="C132" t="str">
         <v/>
       </c>
       <c r="D132">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="133">
@@ -2252,13 +2252,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B133" t="str">
-        <v>TG5GalaxyBlue</v>
+        <v>TG5PerfectAntracit</v>
       </c>
       <c r="C133" t="str">
         <v/>
       </c>
       <c r="D133">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="134">
@@ -2266,7 +2266,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B134" t="str">
-        <v>TG5HollywoodBrown</v>
+        <v>TG5GalaxyBlue</v>
       </c>
       <c r="C134" t="str">
         <v/>
@@ -2280,13 +2280,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B135" t="str">
-        <v>TG5WesternSeaWave</v>
+        <v>TG5HollywoodBrown</v>
       </c>
       <c r="C135" t="str">
         <v/>
       </c>
       <c r="D135">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="136">
@@ -2294,13 +2294,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B136" t="str">
-        <v>TG5EucaliptBZGreen</v>
+        <v>TG5WesternSeaWave</v>
       </c>
       <c r="C136" t="str">
         <v/>
       </c>
       <c r="D136">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="137">
@@ -2308,7 +2308,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B137" t="str">
-        <v>TG5NeonCatsColor</v>
+        <v>TG5EucaliptBZGreen</v>
       </c>
       <c r="C137" t="str">
         <v/>
@@ -2322,13 +2322,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B138" t="str">
-        <v>TG5GraciaBZGreen</v>
+        <v>TG5NeonCatsColor</v>
       </c>
       <c r="C138" t="str">
         <v/>
       </c>
       <c r="D138">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="139">
@@ -2336,13 +2336,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B139" t="str">
-        <v>TG5UrbanBZGray</v>
+        <v>TG5GraciaBZGreen</v>
       </c>
       <c r="C139" t="str">
         <v/>
       </c>
       <c r="D139">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="140">
@@ -2350,13 +2350,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B140" t="str">
-        <v>TG5GraphicaTurq</v>
+        <v>TG5UrbanBZGray</v>
       </c>
       <c r="C140" t="str">
         <v/>
       </c>
       <c r="D140">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="141">
@@ -2364,7 +2364,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B141" t="str">
-        <v>TG5CvetenieGreyBlue</v>
+        <v>TG5GraphicaTurq</v>
       </c>
       <c r="C141" t="str">
         <v/>
@@ -2378,7 +2378,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B142" t="str">
-        <v>TG5ListopadBZgrey</v>
+        <v>TG5PoligonsBlueViol</v>
       </c>
       <c r="C142" t="str">
         <v/>
@@ -2392,13 +2392,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B143" t="str">
-        <v>TG5SymphonyFist</v>
+        <v>TG5CvetenieGreyBlue</v>
       </c>
       <c r="C143" t="str">
         <v/>
       </c>
       <c r="D143">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="144">
@@ -2406,7 +2406,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B144" t="str">
-        <v>TG5MramorGrey</v>
+        <v>TG5VozdSharLightBlue</v>
       </c>
       <c r="C144" t="str">
         <v/>
@@ -2420,7 +2420,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B145" t="str">
-        <v>TG5TatterlineBej</v>
+        <v>TG5YablonevCvetLightBlue</v>
       </c>
       <c r="C145" t="str">
         <v/>
@@ -2434,7 +2434,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B146" t="str">
-        <v>TG5StambulLightBlue</v>
+        <v>TG5PannoGreyTurq</v>
       </c>
       <c r="C146" t="str">
         <v/>
@@ -2448,13 +2448,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B147" t="str">
-        <v>TG5FidgieBZ</v>
+        <v>TG5StambulBej</v>
       </c>
       <c r="C147" t="str">
         <v/>
       </c>
       <c r="D147">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="148">
@@ -2462,13 +2462,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B148" t="str">
-        <v>TG5PoligonsFist</v>
+        <v>TG5NochnoyGorodBordo</v>
       </c>
       <c r="C148" t="str">
         <v/>
       </c>
       <c r="D148">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="149">
@@ -2476,7 +2476,7 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B149" t="str">
-        <v>TG5MishkiTeddiBej</v>
+        <v>TG5AccordBlue</v>
       </c>
       <c r="C149" t="str">
         <v/>
@@ -2490,13 +2490,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B150" t="str">
-        <v>TG5VernisageLightBlue</v>
+        <v>TG5ListopadBZgrey</v>
       </c>
       <c r="C150" t="str">
         <v/>
       </c>
       <c r="D150">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="151">
@@ -2504,13 +2504,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B151" t="str">
-        <v>TG5PoligonsDeepBlue</v>
+        <v>TG5SymphonyFist</v>
       </c>
       <c r="C151" t="str">
         <v/>
       </c>
       <c r="D151">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="152">
@@ -2518,13 +2518,13 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B152" t="str">
-        <v>TG5YablonevCvetPink</v>
+        <v>TG5PannoBejPink</v>
       </c>
       <c r="C152" t="str">
         <v/>
       </c>
       <c r="D152">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="153">
@@ -2532,18 +2532,200 @@
         <v>СЦ (Коляново) (1020002072018000)</v>
       </c>
       <c r="B153" t="str">
+        <v>TG5MramorGrey</v>
+      </c>
+      <c r="C153" t="str">
+        <v/>
+      </c>
+      <c r="D153">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B154" t="str">
+        <v>TG5TatterlineBej</v>
+      </c>
+      <c r="C154" t="str">
+        <v/>
+      </c>
+      <c r="D154">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B155" t="str">
+        <v>TG5StambulLightBlue</v>
+      </c>
+      <c r="C155" t="str">
+        <v/>
+      </c>
+      <c r="D155">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B156" t="str">
+        <v>TG5FidgieBZ</v>
+      </c>
+      <c r="C156" t="str">
+        <v/>
+      </c>
+      <c r="D156">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B157" t="str">
+        <v>TG5AccordTurq</v>
+      </c>
+      <c r="C157" t="str">
+        <v/>
+      </c>
+      <c r="D157">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B158" t="str">
+        <v>TG5AccordViolet</v>
+      </c>
+      <c r="C158" t="str">
+        <v/>
+      </c>
+      <c r="D158">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B159" t="str">
+        <v>TG5PoligonsFist</v>
+      </c>
+      <c r="C159" t="str">
+        <v/>
+      </c>
+      <c r="D159">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B160" t="str">
+        <v>TG5RitmBrown</v>
+      </c>
+      <c r="C160" t="str">
+        <v/>
+      </c>
+      <c r="D160">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B161" t="str">
+        <v>TG5MishkiTeddiBej</v>
+      </c>
+      <c r="C161" t="str">
+        <v/>
+      </c>
+      <c r="D161">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B162" t="str">
+        <v>TG5VernisageLightBlue</v>
+      </c>
+      <c r="C162" t="str">
+        <v/>
+      </c>
+      <c r="D162">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B163" t="str">
+        <v>TG5PoligonsDeepBlue</v>
+      </c>
+      <c r="C163" t="str">
+        <v/>
+      </c>
+      <c r="D163">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B164" t="str">
+        <v>TG5TatterlineFist</v>
+      </c>
+      <c r="C164" t="str">
+        <v/>
+      </c>
+      <c r="D164">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B165" t="str">
+        <v>TG5YablonevCvetPink</v>
+      </c>
+      <c r="C165" t="str">
+        <v/>
+      </c>
+      <c r="D165">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="str">
+        <v>СЦ (Коляново) (1020002072018000)</v>
+      </c>
+      <c r="B166" t="str">
         <v>TG5StambulGreen</v>
       </c>
-      <c r="C153" t="str">
-        <v/>
-      </c>
-      <c r="D153">
+      <c r="C166" t="str">
+        <v/>
+      </c>
+      <c r="D166">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D153"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D166"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>